<commit_message>
Rebuild semantic core: very exact frequency, no zero, two directions only
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016UEhV6w824sjkUhMCvDZb2
</commit_message>
<xml_diff>
--- a/semantic_core_t-ind.ru.xlsx
+++ b/semantic_core_t-ind.ru.xlsx
@@ -9,7 +9,6 @@
   <sheets>
     <sheet name="Шиномонтажное оборудование" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Балансировочные станки" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Примечания" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Шиномонтажное оборудование'!$A$1:$E$101</definedName>
@@ -470,11 +469,11 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>шиномонтажный станок</t>
+          <t>шиномонтажное оборудование</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>44465</v>
+        <v>1140</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -483,23 +482,23 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки</t>
+          <t>Шиномонтажное оборудование (общие)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki</t>
+          <t>/catalog/shinomontazhnoe-oborudovanie</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>шиномонтажное оборудование</t>
+          <t>шиномонтажный станок</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>13734</v>
+        <v>1005</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -508,23 +507,23 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование (общие)</t>
+          <t>Шиномонтажные станки</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>/catalog/shinomontazhnye-stanki</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>шиномонтажный станок купить</t>
+          <t>шиномонтажное оборудование купить</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>6299</v>
+        <v>542</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -533,23 +532,23 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки</t>
+          <t>Шиномонтажное оборудование (общие)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki</t>
+          <t>/catalog/shinomontazhnoe-oborudovanie</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>шиномонтажное оборудование купить</t>
+          <t>ручной шиномонтажный станок</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>4533</v>
+        <v>479</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -558,23 +557,23 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование (общие)</t>
+          <t>Ручные шиномонтажные станки</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>грузовой шиномонтажный станок</t>
+          <t>шиномонтажный станок купить</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>3320</v>
+        <v>436</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -583,23 +582,23 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки для грузовых</t>
+          <t>Шиномонтажные станки</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki-dlya-gruzovyh-avtomobilej</t>
+          <t>/catalog/shinomontazhnye-stanki</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>сивик шиномонтажное</t>
+          <t>вулканизатор для шиномонтажа</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2848</v>
+        <v>324</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -608,23 +607,23 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование по брендам</t>
+          <t>Вулканизаторы и ремонт шин</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie/brand-sivik</t>
+          <t>/catalog/vulkanizatory</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>клей для вулканизации</t>
+          <t>сивик шиномонтажное оборудование официальный сайт</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>2129</v>
+        <v>273</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -633,23 +632,23 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Вулканизаторы и ремонт шин</t>
+          <t>Шиномонтажное оборудование по брендам</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>/catalog/vulkanizatory</t>
+          <t>/catalog/shinomontazhnoe-oborudovanie/brand-sivik</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>шиномонтажный стенд</t>
+          <t>сивик шиномонтажное оборудование</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>2000</v>
+        <v>239</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -658,23 +657,23 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки</t>
+          <t>Шиномонтажное оборудование по брендам</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki</t>
+          <t>/catalog/shinomontazhnoe-oborudovanie/brand-sivik</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ручной шиномонтажный станок</t>
+          <t>клей активатор для холодной вулканизации</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>1951</v>
+        <v>225</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -683,23 +682,23 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Ручные шиномонтажные станки</t>
+          <t>Вулканизаторы и ремонт шин</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej</t>
+          <t>/catalog/vulkanizatory</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>шиномонтажный станок сивик</t>
+          <t>оборудование для шиномонтажа комплект цена</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>1809</v>
+        <v>214</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -708,23 +707,23 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование по брендам</t>
+          <t>Комплекты и инструмент для шиномонтажа</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie/brand-sivik</t>
+          <t>/catalog/komplekty-shinomontazhnogo-oborudovaniya</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>купить станки для шиномонтажа</t>
+          <t>ручной шиномонтажный станок купить для дома</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>1778</v>
+        <v>202</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -733,23 +732,23 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование (общие)</t>
+          <t>Ручные шиномонтажные станки</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>вулканизатор купить</t>
+          <t>шиномонтажное оборудование комплект</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>1742</v>
+        <v>178</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -758,23 +757,23 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Вулканизаторы и ремонт шин</t>
+          <t>Комплекты и инструмент для шиномонтажа</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>/catalog/vulkanizatory</t>
+          <t>/catalog/komplekty-shinomontazhnogo-oborudovaniya</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>шиномонтажный комплект</t>
+          <t>шиномонтажный станок сивик</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>1695</v>
+        <v>158</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -783,23 +782,23 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Комплекты и инструмент для шиномонтажа</t>
+          <t>Шиномонтажное оборудование по брендам</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>/catalog/komplekty-shinomontazhnogo-oborudovaniya</t>
+          <t>/catalog/shinomontazhnoe-oborudovanie/brand-sivik</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>станок шиномонтажный легковой</t>
+          <t>борторасширитель для шиномонтажа</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>1681</v>
+        <v>138</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -808,23 +807,23 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки для легковых</t>
+          <t>Шиномонтажное оборудование (общие)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej</t>
+          <t>/catalog/shinomontazhnoe-oborudovanie</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>шиномонтажный станок нордберг</t>
+          <t>грузовой шиномонтажный станок</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>1630</v>
+        <v>130</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -833,23 +832,23 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование по брендам</t>
+          <t>Шиномонтажные станки для грузовых</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie/brand-nordberg</t>
+          <t>/catalog/shinomontazhnye-stanki-dlya-gruzovyh-avtomobilej</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>клей для холодной вулканизации</t>
+          <t>станок шиномонтажный легковой</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>1491</v>
+        <v>128</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -858,23 +857,23 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Вулканизаторы и ремонт шин</t>
+          <t>Шиномонтажные станки для легковых</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>/catalog/vulkanizatory</t>
+          <t>/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>вулканизатор камер</t>
+          <t>оборудование для грузового шиномонтажа</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>1265</v>
+        <v>123</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -883,23 +882,23 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Вулканизаторы и ремонт шин</t>
+          <t>Шиномонтажные станки для грузовых</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>/catalog/vulkanizatory</t>
+          <t>/catalog/shinomontazhnye-stanki-dlya-gruzovyh-avtomobilej</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>запчасти шиномонтажного станка</t>
+          <t>rossvik шиномонтажное оборудование</t>
         </is>
       </c>
       <c r="B19" t="n">
-        <v>1215</v>
+        <v>103</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -908,23 +907,23 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Запчасти для шиномонтажных станков</t>
+          <t>Шиномонтажное оборудование по брендам</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>/catalog/rashodnye-materialy-dlya-shinomontazhnogo-oborudovaniya</t>
+          <t>/catalog/shinomontazhnoe-oborudovanie</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>шиномонтажное оборудование комплект</t>
+          <t>станок шиномонтажный легковой купить</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>1188</v>
+        <v>97</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -933,23 +932,23 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Комплекты и инструмент для шиномонтажа</t>
+          <t>Шиномонтажные станки для легковых</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>/catalog/komplekty-shinomontazhnogo-oborudovaniya</t>
+          <t>/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>грузовой шиномонтаж купить</t>
+          <t>клей для холодной вулканизации</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>950</v>
+        <v>97</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -958,23 +957,23 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки для грузовых</t>
+          <t>Вулканизаторы и ремонт шин</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki-dlya-gruzovyh-avtomobilej</t>
+          <t>/catalog/vulkanizatory</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>шиномонтажные станки сивик</t>
+          <t>монтировка для шиномонтажа</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>936</v>
+        <v>92</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -983,23 +982,23 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование по брендам</t>
+          <t>Шиномонтажное оборудование (общие)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie/brand-sivik</t>
+          <t>/catalog/shinomontazhnoe-oborudovanie</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ручной шиномонтаж</t>
+          <t>вулканизатор купить</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>933</v>
+        <v>88</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1008,23 +1007,23 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Ручные шиномонтажные станки</t>
+          <t>Вулканизаторы и ремонт шин</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej</t>
+          <t>/catalog/vulkanizatory</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>домкрат для шиномонтажа</t>
+          <t>шиномонтажный станок нордберг</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>903</v>
+        <v>84</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1033,23 +1032,23 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Подъемники и домкраты для шиномонтажа</t>
+          <t>Шиномонтажное оборудование по брендам</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>/catalog/shinomontazhnoe-oborudovanie/brand-nordberg</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>сивик шиномонтажное оборудование</t>
+          <t>инструмент для шиномонтажа</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>889</v>
+        <v>81</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1058,23 +1057,23 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование по брендам</t>
+          <t>Комплекты и инструмент для шиномонтажа</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie/brand-sivik</t>
+          <t>/catalog/komplekty-shinomontazhnogo-oborudovaniya</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>вулканизатор шин</t>
+          <t>латки для шиномонтажа</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>867</v>
+        <v>71</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1095,11 +1094,11 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>шиномонтажный станок автомат</t>
+          <t>ручной шиномонтаж</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>834</v>
+        <v>70</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1108,23 +1107,23 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Автоматические шиномонтажные станки</t>
+          <t>Ручные шиномонтажные станки</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki/vid-avtomaticheskij</t>
+          <t>/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>вулканизатор для ремонта</t>
+          <t>шиномонтаж hunter</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>830</v>
+        <v>68</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1133,23 +1132,23 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Вулканизаторы и ремонт шин</t>
+          <t>Шиномонтажное оборудование по брендам</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>/catalog/vulkanizatory</t>
+          <t>/catalog/shinomontazhnoe-oborudovanie/brand-hunterengineering</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>мойка для шиномонтажа</t>
+          <t>купить оборудование для шиномонтажа легковых автомобилей</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>829</v>
+        <v>66</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1158,23 +1157,23 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Мойки колес</t>
+          <t>Шиномонтажные станки для легковых</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>/catalog/mojki-koles</t>
+          <t>/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>вулканизатор для шиномонтажа</t>
+          <t>ручной шиномонтажный станок купить</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>826</v>
+        <v>65</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1183,23 +1182,23 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Вулканизаторы и ремонт шин</t>
+          <t>Ручные шиномонтажные станки</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>/catalog/vulkanizatory</t>
+          <t>/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>инструмент для шиномонтажа</t>
+          <t>заплатки для шиномонтажа купить</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>783</v>
+        <v>64</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1208,23 +1207,23 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Комплекты и инструмент для шиномонтажа</t>
+          <t>Вулканизаторы и ремонт шин</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>/catalog/komplekty-shinomontazhnogo-oborudovaniya</t>
+          <t>/catalog/vulkanizatory</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>подъемник для шиномонтажа</t>
+          <t>вулканизатор россвик</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>769</v>
+        <v>62</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -1233,23 +1232,23 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Подъемники и домкраты для шиномонтажа</t>
+          <t>Вулканизаторы и ремонт шин</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>/catalog/vulkanizatory</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>мойка колес для шиномонтажа</t>
+          <t>третья рука для шиномонтажного станка</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>725</v>
+        <v>62</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -1258,23 +1257,23 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Мойки колес</t>
+          <t>Шиномонтажное оборудование (общие)</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>/catalog/mojki-koles</t>
+          <t>/catalog/shinomontazhnoe-oborudovanie</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>россвик шиномонтажное</t>
+          <t>вулканизатор для камер</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>719</v>
+        <v>61</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -1283,23 +1282,23 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование по брендам</t>
+          <t>Вулканизаторы и ремонт шин</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>/catalog/vulkanizatory</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>шиномонтажный станок для легковых автомобилей</t>
+          <t>бустер для шиномонтажа</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>675</v>
+        <v>59</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -1308,23 +1307,23 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки для легковых</t>
+          <t>Шиномонтажное оборудование (общие)</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej</t>
+          <t>/catalog/shinomontazhnoe-oborudovanie</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>клей активатор для холодной вулканизации</t>
+          <t>шиномонтажное оборудование купить в новосибирске</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>652</v>
+        <v>57</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1333,23 +1332,23 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Вулканизаторы и ремонт шин</t>
+          <t>Шиномонтажное оборудование (общие)</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>/catalog/vulkanizatory</t>
+          <t>/catalog/shinomontazhnoe-oborudovanie</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>станок шиномонтажный легковой купить</t>
+          <t>клей для латок шиномонтажный</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>650</v>
+        <v>54</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1358,23 +1357,23 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки для легковых</t>
+          <t>Вулканизаторы и ремонт шин</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej</t>
+          <t>/catalog/vulkanizatory</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>вулканизатор комплекс</t>
+          <t>мыло для шиномонтажа</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>623</v>
+        <v>54</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1383,23 +1382,23 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Вулканизаторы и ремонт шин</t>
+          <t>Шиномонтажное оборудование (общие)</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>/catalog/vulkanizatory</t>
+          <t>/catalog/shinomontazhnoe-oborudovanie</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>материалы для шиномонтажа</t>
+          <t>шиномонтажный стенд</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>615</v>
+        <v>54</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -1408,23 +1407,23 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование (общие)</t>
+          <t>Шиномонтажные станки</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>/catalog/shinomontazhnye-stanki</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>шиномонтажное оборудование цена</t>
+          <t>вулканизатор для грузовых шин</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>611</v>
+        <v>53</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -1433,23 +1432,23 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование (общие)</t>
+          <t>Вулканизаторы и ремонт шин</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>/catalog/vulkanizatory</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>купить грузовой шиномонтажный станок</t>
+          <t>шиномонтажное оборудование комплект купить цена</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>590</v>
+        <v>50</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -1458,23 +1457,23 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки для грузовых</t>
+          <t>Комплекты и инструмент для шиномонтажа</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki-dlya-gruzovyh-avtomobilej</t>
+          <t>/catalog/komplekty-shinomontazhnogo-oborudovaniya</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>третья рука шиномонтажного станка</t>
+          <t>автоматический шиномонтажный станок</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>581</v>
+        <v>48</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -1483,23 +1482,23 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование (общие)</t>
+          <t>Автоматические шиномонтажные станки</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>/catalog/shinomontazhnye-stanki/vid-avtomaticheskij</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>оборудование для грузового шиномонтажа</t>
+          <t>ванна для шиномонтажа</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>562</v>
+        <v>48</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -1508,23 +1507,23 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки для грузовых</t>
+          <t>Шиномонтажное оборудование (общие)</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki-dlya-gruzovyh-avtomobilej</t>
+          <t>/catalog/shinomontazhnoe-oborudovanie</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>монтировка для шиномонтажа</t>
+          <t>расширитель шин для шиномонтажа</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>541</v>
+        <v>45</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -1545,11 +1544,11 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>шиномонтажный станок 220в</t>
+          <t>шиномонтажный станок для легковых автомобилей</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>538</v>
+        <v>44</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -1558,23 +1557,23 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки</t>
+          <t>Шиномонтажные станки для легковых</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki</t>
+          <t>/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>шиномонтажный стол</t>
+          <t>станок для шиномонтажа грузовых автомобилей</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>537</v>
+        <v>43</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -1583,23 +1582,23 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование (общие)</t>
+          <t>Шиномонтажные станки для грузовых</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>/catalog/shinomontazhnye-stanki-dlya-gruzovyh-avtomobilej</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>ручной шиномонтажный станок купить</t>
+          <t>шиномонтажный станок хоффман</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>529</v>
+        <v>42</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -1608,23 +1607,23 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Ручные шиномонтажные станки</t>
+          <t>Шиномонтажное оборудование по брендам</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej</t>
+          <t>/catalog/shinomontazhnoe-oborudovanie</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>вулканизатор грузовой</t>
+          <t>шиномонтажное оборудование купить в иркутске</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>507</v>
+        <v>41</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -1633,23 +1632,23 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Вулканизаторы и ремонт шин</t>
+          <t>Шиномонтажное оборудование (общие)</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>/catalog/vulkanizatory</t>
+          <t>/catalog/shinomontazhnoe-oborudovanie</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>шиномонтажный станок полуавтоматический</t>
+          <t>шиномонтажное оборудование купить в москве</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>496</v>
+        <v>41</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
@@ -1658,23 +1657,23 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Автоматические шиномонтажные станки</t>
+          <t>Шиномонтажное оборудование (общие)</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki/vid-poluavtomaticheskij</t>
+          <t>/catalog/shinomontazhnoe-oborudovanie</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>накладки на шиномонтажный станок</t>
+          <t>nordberg шиномонтажное оборудование</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>478</v>
+        <v>39</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
@@ -1683,23 +1682,23 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки</t>
+          <t>Шиномонтажное оборудование по брендам</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki</t>
+          <t>/catalog/shinomontazhnoe-oborudovanie/brand-nordberg</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>домкрат подкатной для шиномонтажа</t>
+          <t>шиномонтаж под ключ</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>477</v>
+        <v>37</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
@@ -1708,7 +1707,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Подъемники и домкраты для шиномонтажа</t>
+          <t>Шиномонтажное оборудование (общие)</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -1720,11 +1719,11 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>шиномонтажное оборудование официальный сайт</t>
+          <t>габариты шиномонтажного станка</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>474</v>
+        <v>37</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
@@ -1745,11 +1744,11 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>шиномонтажный магазин</t>
+          <t>шиномонтажное оборудование комплект купить</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>470</v>
+        <v>37</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
@@ -1758,23 +1757,23 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование (общие)</t>
+          <t>Комплекты и инструмент для шиномонтажа</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>/catalog/komplekty-shinomontazhnogo-oborudovaniya</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>оборудование для шиномонтажа комплект цена</t>
+          <t>шиномонтаж оборудование цены полный комплект</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>453</v>
+        <v>37</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
@@ -1795,11 +1794,11 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>купить легковой шиномонтаж</t>
+          <t>инструменты для шиномонтажа купить</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>446</v>
+        <v>36</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
@@ -1808,23 +1807,23 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки для легковых</t>
+          <t>Комплекты и инструмент для шиномонтажа</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej</t>
+          <t>/catalog/komplekty-shinomontazhnogo-oborudovaniya</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>шиномонтажный комплект купить</t>
+          <t>монтажная лопатка для шиномонтажа</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>441</v>
+        <v>36</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
@@ -1833,23 +1832,23 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Комплекты и инструмент для шиномонтажа</t>
+          <t>Шиномонтажное оборудование (общие)</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>/catalog/komplekty-shinomontazhnogo-oborudovaniya</t>
+          <t>/catalog/shinomontazhnoe-oborudovanie</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>педаль шиномонтажного станка</t>
+          <t>лифт для колес на шиномонтаж</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>434</v>
+        <v>36</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
@@ -1870,11 +1869,11 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>шиномонтажный станок характеристики</t>
+          <t>гайковерт электрический для шиномонтажа</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>405</v>
+        <v>35</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
@@ -1883,23 +1882,23 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки</t>
+          <t>Шиномонтажное оборудование (общие)</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki</t>
+          <t>/catalog/shinomontazhnoe-oborudovanie</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>шиномонтажный станок хоффман</t>
+          <t>масло для шиномонтажного станка</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>360</v>
+        <v>35</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
@@ -1908,7 +1907,7 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование по брендам</t>
+          <t>Шиномонтажное оборудование (общие)</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -1920,11 +1919,11 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>сивик шиномонтажное оборудование официальный</t>
+          <t>шиномонтажное оборудование 220 вольт</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>346</v>
+        <v>35</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
@@ -1933,23 +1932,23 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование по брендам</t>
+          <t>Шиномонтажное оборудование (общие)</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie/brand-sivik</t>
+          <t>/catalog/shinomontazhnoe-oborudovanie</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>шиномонтажное оборудование сивик официальный сайт</t>
+          <t>шиномонтажное оборудование цена</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>345</v>
+        <v>34</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
@@ -1958,23 +1957,23 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование по брендам</t>
+          <t>Шиномонтажное оборудование (общие)</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie/brand-sivik</t>
+          <t>/catalog/shinomontazhnoe-oborudovanie</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>стол шиномонтажного станка</t>
+          <t>купить грузовой шиномонтажный станок</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>343</v>
+        <v>33</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
@@ -1983,23 +1982,23 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование (общие)</t>
+          <t>Шиномонтажные станки для грузовых</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>/catalog/shinomontazhnye-stanki-dlya-gruzovyh-avtomobilej</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>магазин шиномонтажного оборудования</t>
+          <t>купить шиномонтажный станок для легковых автомобилей</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>341</v>
+        <v>33</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
@@ -2008,23 +2007,23 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование (общие)</t>
+          <t>Шиномонтажные станки для легковых</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>станок шиномонтажный для грузовых автомобилей</t>
+          <t>магазин шиномонтажного оборудования</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>341</v>
+        <v>33</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
@@ -2033,23 +2032,23 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки для грузовых</t>
+          <t>Шиномонтажное оборудование (общие)</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki-dlya-gruzovyh-avtomobilej</t>
+          <t>/catalog/shinomontazhnoe-oborudovanie</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>стенд шиномонтажный грузовой</t>
+          <t>оборудование для шиномонтажа комплект под ключ цена</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>333</v>
+        <v>32</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
@@ -2058,23 +2057,23 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки для грузовых</t>
+          <t>Комплекты и инструмент для шиномонтажа</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki-dlya-gruzovyh-avtomobilej</t>
+          <t>/catalog/komplekty-shinomontazhnogo-oborudovaniya</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>шиномонтажный станок kraftwell</t>
+          <t>грузовой шиномонтаж купить</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>330</v>
+        <v>30</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
@@ -2083,23 +2082,23 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование по брендам</t>
+          <t>Шиномонтажные станки для грузовых</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>/catalog/shinomontazhnye-stanki-dlya-gruzovyh-avtomobilej</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>шиномонтаж нордберг</t>
+          <t>третья рука для шиномонтажного станка купить</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>329</v>
+        <v>30</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
@@ -2108,23 +2107,23 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование по брендам</t>
+          <t>Шиномонтажное оборудование (общие)</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie/brand-nordberg</t>
+          <t>/catalog/shinomontazhnoe-oborudovanie</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>шиномонтажное оборудование комплект купить</t>
+          <t>купить оборудование для грузового шиномонтажа</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>327</v>
+        <v>30</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
@@ -2133,23 +2132,23 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Комплекты и инструмент для шиномонтажа</t>
+          <t>Шиномонтажные станки для грузовых</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>/catalog/komplekty-shinomontazhnogo-oborudovaniya</t>
+          <t>/catalog/shinomontazhnye-stanki-dlya-gruzovyh-avtomobilej</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>шиномонтажное оборудование для легковых автомобилей</t>
+          <t>станок разбортовочный для шиномонтажа</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>311</v>
+        <v>29</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
@@ -2158,23 +2157,23 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки для легковых</t>
+          <t>Шиномонтажные станки</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej</t>
+          <t>/catalog/shinomontazhnye-stanki</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>купить шиномонтажное оборудование для легковых автомобилей</t>
+          <t>шиномонтажный станок нордберг 4638е</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>310</v>
+        <v>29</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
@@ -2183,23 +2182,23 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки для легковых</t>
+          <t>Шиномонтажное оборудование по брендам</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej</t>
+          <t>/catalog/shinomontazhnoe-oborudovanie/brand-nordberg</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>все для шиномонтажа магазин</t>
+          <t>купить шиномонтажное оборудование для легковых автомобилей новое</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>275</v>
+        <v>28</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
@@ -2208,23 +2207,23 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование (общие)</t>
+          <t>Шиномонтажные станки для легковых</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>станок шиномонтажный цена</t>
+          <t>монтировка для шиномонтажа грузовых автомобилей</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>263</v>
+        <v>28</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
@@ -2233,23 +2232,23 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки</t>
+          <t>Шиномонтажные станки для грузовых</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki</t>
+          <t>/catalog/shinomontazhnye-stanki-dlya-gruzovyh-avtomobilej</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>шиномонтаж под ключ</t>
+          <t>сибек оборудование для шиномонтажа</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>259</v>
+        <v>28</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
@@ -2270,11 +2269,11 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>купить шиномонтажный станок для легковых автомобилей</t>
+          <t>вес шиномонтажного станка</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>254</v>
+        <v>27</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
@@ -2283,23 +2282,23 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки для легковых</t>
+          <t>Шиномонтажное оборудование (общие)</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej</t>
+          <t>/catalog/shinomontazhnoe-oborudovanie</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>домкрат для шиномонтажа купить</t>
+          <t>шиномонтажный станок kraftwell</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>242</v>
+        <v>27</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
@@ -2308,7 +2307,7 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Подъемники и домкраты для шиномонтажа</t>
+          <t>Шиномонтажное оборудование по брендам</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
@@ -2320,11 +2319,11 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>шиномонтажный станок техносоюз</t>
+          <t>оборудование для шиномонтажа купить в спб</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>237</v>
+        <v>27</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
@@ -2333,7 +2332,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование по брендам</t>
+          <t>Шиномонтажное оборудование (общие)</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -2345,11 +2344,11 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>нордберг шиномонтажное оборудование</t>
+          <t>шиномонтажное оборудование в рассрочку</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>233</v>
+        <v>27</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
@@ -2358,23 +2357,23 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование по брендам</t>
+          <t>Шиномонтажное оборудование (общие)</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie/brand-nordberg</t>
+          <t>/catalog/shinomontazhnoe-oborudovanie</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>лучшее шиномонтажное оборудование</t>
+          <t>все для шиномонтажа магазин</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>233</v>
+        <v>27</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
@@ -2395,11 +2394,11 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>шиномонтажный станок кс 302а</t>
+          <t>шиномонтажный комплект</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>231</v>
+        <v>26</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
@@ -2408,23 +2407,23 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки</t>
+          <t>Комплекты и инструмент для шиномонтажа</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki</t>
+          <t>/catalog/komplekty-shinomontazhnogo-oborudovaniya</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>купить шиномонтажный станок сивик</t>
+          <t>расширитель бортов для шиномонтажа</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>222</v>
+        <v>26</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
@@ -2433,23 +2432,23 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование по брендам</t>
+          <t>Шиномонтажное оборудование (общие)</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie/brand-sivik</t>
+          <t>/catalog/shinomontazhnoe-oborudovanie</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>набор шиномонтажный</t>
+          <t>станок шиномонтажный легковой автоматический 220в</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>215</v>
+        <v>26</v>
       </c>
       <c r="C81" t="inlineStr">
         <is>
@@ -2458,23 +2457,23 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Комплекты и инструмент для шиномонтажа</t>
+          <t>Шиномонтажные станки для легковых</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>/catalog/komplekty-shinomontazhnogo-oborudovaniya</t>
+          <t>/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>шиномонтаж hunter</t>
+          <t>кс 302а шиномонтажный станок sivik</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>213</v>
+        <v>26</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
@@ -2488,18 +2487,18 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie/brand-hunterengineering</t>
+          <t>/catalog/shinomontazhnoe-oborudovanie/brand-sivik</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>ручной шиномонтажный станок купить для дома</t>
+          <t>автоматическая подкачка колес для шиномонтажа</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>209</v>
+        <v>26</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
@@ -2508,23 +2507,23 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Ручные шиномонтажные станки</t>
+          <t>Автоматические шиномонтажные станки</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej</t>
+          <t>/catalog/shinomontazhnye-stanki/vid-avtomaticheskij</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>ножничный подъемник для шиномонтажа</t>
+          <t>шиномонтажные станки для легковых авто</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>209</v>
+        <v>26</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
@@ -2533,23 +2532,23 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Подъемники и домкраты для шиномонтажа</t>
+          <t>Шиномонтажные станки для легковых</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>оборудование под шиномонтаж</t>
+          <t>материалы для шиномонтажа</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>208</v>
+        <v>25</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
@@ -2570,11 +2569,11 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>шиномонтажный станок троммельберг</t>
+          <t>шиномонтажный станок нордберг 4638</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>207</v>
+        <v>25</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
@@ -2588,18 +2587,18 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>/catalog/shinomontazhnoe-oborudovanie/brand-nordberg</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>борторасширитель для шиномонтажа</t>
+          <t>eqfs шиномонтажный станок</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>206</v>
+        <v>25</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
@@ -2608,23 +2607,23 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование (общие)</t>
+          <t>Шиномонтажные станки</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>/catalog/shinomontazhnye-stanki</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>шиномонтажный станок нордберг 4638е</t>
+          <t>шиномонтажное оборудование воронеж</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>198</v>
+        <v>25</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
@@ -2633,48 +2632,48 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование по брендам</t>
+          <t>Шиномонтажное оборудование (общие)</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie/brand-nordberg</t>
+          <t>/catalog/shinomontazhnoe-oborudovanie</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>устройство шиномонтажного станка</t>
+          <t>шиномонтажный станок сивик кс 402а про</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>191</v>
+        <v>25</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Информационный</t>
+          <t>Коммерческий</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование (общие)</t>
+          <t>Шиномонтажное оборудование по брендам</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>/catalog/shinomontazhnoe-oborudovanie/brand-sivik</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>станкоимпорт шиномонтажный станок</t>
+          <t>китайский шиномонтажный станок</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>186</v>
+        <v>24</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
@@ -2683,23 +2682,23 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование по брендам</t>
+          <t>Шиномонтажные станки</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>/catalog/shinomontazhnye-stanki</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>ванна для шиномонтажа</t>
+          <t>генератор азота для шиномонтажа</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>186</v>
+        <v>24</v>
       </c>
       <c r="C91" t="inlineStr">
         <is>
@@ -2724,7 +2723,7 @@
         </is>
       </c>
       <c r="B92" t="n">
-        <v>185</v>
+        <v>24</v>
       </c>
       <c r="C92" t="inlineStr">
         <is>
@@ -2745,11 +2744,11 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>купить шиномонтаж в спб</t>
+          <t>шиномонтажный станок суперавтомат кс 508а про</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>185</v>
+        <v>24</v>
       </c>
       <c r="C93" t="inlineStr">
         <is>
@@ -2758,23 +2757,23 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование (общие)</t>
+          <t>Автоматические шиномонтажные станки</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>/catalog/shinomontazhnye-stanki/vid-avtomaticheskij</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>подкатной домкрат для шиномонтажа профессиональный</t>
+          <t>крафтвелл шиномонтажное оборудование</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>179</v>
+        <v>24</v>
       </c>
       <c r="C94" t="inlineStr">
         <is>
@@ -2783,7 +2782,7 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Подъемники и домкраты для шиномонтажа</t>
+          <t>Шиномонтажное оборудование по брендам</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -2795,11 +2794,11 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>россвик шиномонтажное оборудование</t>
+          <t>хантер шиномонтажное оборудование</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>179</v>
+        <v>24</v>
       </c>
       <c r="C95" t="inlineStr">
         <is>
@@ -2813,18 +2812,18 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>/catalog/shinomontazhnoe-oborudovanie/brand-hunterengineering</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>шиномонтажное оборудование в новосибирске</t>
+          <t>купить станки для шиномонтажа</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>179</v>
+        <v>23</v>
       </c>
       <c r="C96" t="inlineStr">
         <is>
@@ -2845,11 +2844,11 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>eqfs шиномонтажный станок</t>
+          <t>шиномонтажный станок с 3 рукой</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>178</v>
+        <v>23</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
@@ -2870,11 +2869,11 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>продажа шиномонтажного оборудования</t>
+          <t>ключ третья рука</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>178</v>
+        <v>22</v>
       </c>
       <c r="C98" t="inlineStr">
         <is>
@@ -2895,11 +2894,11 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>третья рука сивик</t>
+          <t>комплект шиномонтажного оборудования для легковых автомобилей цена</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>177</v>
+        <v>22</v>
       </c>
       <c r="C99" t="inlineStr">
         <is>
@@ -2908,23 +2907,23 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование по брендам</t>
+          <t>Комплекты и инструмент для шиномонтажа</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie/brand-sivik</t>
+          <t>/catalog/komplekty-shinomontazhnogo-oborudovaniya</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>пневматический шиномонтажный станок</t>
+          <t>сколько весит шиномонтажный станок</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>176</v>
+        <v>22</v>
       </c>
       <c r="C100" t="inlineStr">
         <is>
@@ -2945,11 +2944,11 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>масло для шиномонтажного станка</t>
+          <t>конус для шиномонтажного станка на газель</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>175</v>
+        <v>22</v>
       </c>
       <c r="C101" t="inlineStr">
         <is>
@@ -3023,7 +3022,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>30508</v>
+        <v>459</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -3044,11 +3043,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>балансировочный станок сивик</t>
+          <t>балансировочный станок для шиномонтажа</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>2994</v>
+        <v>279</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -3057,23 +3056,23 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировка в составе шиномонтажного оборудования</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-sivik</t>
+          <t>/catalog/balansirovochnye-stanki</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>балансировочный станок для шиномонтажа</t>
+          <t>балансировочный станок для шиномонтажа купить</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>2014</v>
+        <v>205</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -3094,11 +3093,11 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>балансировочный станок нордберг</t>
+          <t>балансировочный станок sivik</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>950</v>
+        <v>136</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -3112,7 +3111,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-nordberg</t>
+          <t>/catalog/balansirovochnye-stanki/brand-sivik</t>
         </is>
       </c>
     </row>
@@ -3123,7 +3122,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>851</v>
+        <v>67</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -3148,7 +3147,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>727</v>
+        <v>65</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -3169,11 +3168,11 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>стенд для балансировки</t>
+          <t>аппарат для балансировки колес</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>726</v>
+        <v>59</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -3194,11 +3193,11 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>балансировочный станок для шиномонтажа купить</t>
+          <t>балансировочный станок нордберг</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>627</v>
+        <v>46</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -3207,23 +3206,23 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Балансировка в составе шиномонтажного оборудования</t>
+          <t>Балансировочные станки по брендам</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>/catalog/balansirovochnye-stanki/brand-nordberg</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>балансировка колес купить</t>
+          <t>стенд для балансировки колес</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>572</v>
+        <v>38</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -3244,11 +3243,11 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>балансировочный станок россвик</t>
+          <t>фланцевый адаптер для балансировки колес</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>478</v>
+        <v>37</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -3257,7 +3256,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировочные станки (общие)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -3269,11 +3268,11 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>купить балансировочный станок сивик</t>
+          <t>балансировочный станок hunter</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>397</v>
+        <v>37</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -3287,18 +3286,18 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-sivik</t>
+          <t>/catalog/balansirovochnye-stanki/brand-hunterengineering</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>станок балансировочный легковой</t>
+          <t>купить балансировочный станок сивик</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>377</v>
+        <v>35</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -3307,23 +3306,23 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Балансировочные станки для легковых</t>
+          <t>Балансировочные станки по брендам</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki-dlya-legkovyh-avtomobilej</t>
+          <t>/catalog/balansirovochnye-stanki/brand-sivik</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>станок для балансировки купить</t>
+          <t>оборудование для балансировки колес</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>345</v>
+        <v>34</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -3344,11 +3343,11 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>балансировочный станок kraftwell</t>
+          <t>балансировочный станок с нагрузочным роликом</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>342</v>
+        <v>29</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -3357,7 +3356,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировочные станки (общие)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -3369,11 +3368,11 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>адаптер для балансировки колес</t>
+          <t>приспособление для балансировки колес</t>
         </is>
       </c>
       <c r="B16" t="n">
-        <v>333</v>
+        <v>25</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -3394,11 +3393,11 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>сторм станок балансировочный</t>
+          <t>балансировочный станок для шиномонтажа сивик</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>333</v>
+        <v>24</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -3412,18 +3411,18 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-storm</t>
+          <t>/catalog/balansirovochnye-stanki/brand-sivik</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>конус для балансировки колес</t>
+          <t>балансировочный станок sivik galaxy</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>312</v>
+        <v>23</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -3432,12 +3431,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировочные станки по брендам</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>/catalog/balansirovochnye-stanki/brand-sivik</t>
         </is>
       </c>
     </row>
@@ -3448,7 +3447,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>294</v>
+        <v>23</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -3469,11 +3468,11 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>балансировочный станок hofmann</t>
+          <t>микробисер для балансировки колес</t>
         </is>
       </c>
       <c r="B20" t="n">
-        <v>279</v>
+        <v>23</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -3482,7 +3481,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировочные станки (общие)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -3494,20 +3493,20 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>балансировочный станок galaxy plus</t>
+          <t>устройство для балансировки колес</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>257</v>
+        <v>23</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Коммерческий</t>
+          <t>Информационный</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировочные станки (общие)</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -3519,11 +3518,11 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>балансировочный станок сивик галакси</t>
+          <t>сторм балансировочный станок</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>247</v>
+        <v>23</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -3537,18 +3536,18 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-sivik</t>
+          <t>/catalog/balansirovochnye-stanki/brand-storm</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>самоклеющиеся балансировочные грузики</t>
+          <t>сивик гелиос балансировочный станок</t>
         </is>
       </c>
       <c r="B23" t="n">
-        <v>243</v>
+        <v>23</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -3557,23 +3556,23 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Балансировочные грузики</t>
+          <t>Балансировочные станки по брендам</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>/catalog/gruziki-balansirovochnye</t>
+          <t>/catalog/balansirovochnye-stanki/brand-sivik</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>балансировочный станок hunter</t>
+          <t>балансировочный станок nordberg 4523c</t>
         </is>
       </c>
       <c r="B24" t="n">
-        <v>236</v>
+        <v>22</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -3587,18 +3586,18 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-hunterengineering</t>
+          <t>/catalog/balansirovochnye-stanki/brand-nordberg</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>стенд для балансировки колес</t>
+          <t>балансировочный станок для шиномонтажа цена</t>
         </is>
       </c>
       <c r="B25" t="n">
-        <v>228</v>
+        <v>20</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -3607,7 +3606,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировка в составе шиномонтажного оборудования</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -3619,11 +3618,11 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>балансировочный станок автоматический</t>
+          <t>балансировочный станок kraftwell krw242</t>
         </is>
       </c>
       <c r="B26" t="n">
-        <v>222</v>
+        <v>19</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -3632,7 +3631,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Автоматические балансировочные станки</t>
+          <t>Балансировочные станки по брендам</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -3644,11 +3643,11 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ts 500 балансировочный станок</t>
+          <t>стенд для балансировки</t>
         </is>
       </c>
       <c r="B27" t="n">
-        <v>217</v>
+        <v>19</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -3669,11 +3668,11 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>балансировочный станок гелиос</t>
+          <t>балансировочный станок sicam</t>
         </is>
       </c>
       <c r="B28" t="n">
-        <v>195</v>
+        <v>17</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -3694,11 +3693,11 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>балансировочный станок троммельберг</t>
+          <t>купить станок для балансировки колес легковых автомобилей</t>
         </is>
       </c>
       <c r="B29" t="n">
-        <v>184</v>
+        <v>17</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -3707,23 +3706,23 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировочные станки для легковых</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>/catalog/balansirovochnye-stanki-dlya-legkovyh-avtomobilej</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>балансировочный станок civic</t>
+          <t>балансировочный станок троммельберг</t>
         </is>
       </c>
       <c r="B30" t="n">
-        <v>173</v>
+        <v>17</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -3732,7 +3731,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировочные станки по брендам</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -3744,11 +3743,11 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>балансировочный станок vt 63</t>
+          <t>балансировочный станок сивик галакси плюс</t>
         </is>
       </c>
       <c r="B31" t="n">
-        <v>161</v>
+        <v>17</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -3757,23 +3756,23 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировочные станки по брендам</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>/catalog/balansirovochnye-stanki/brand-sivik</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>сивик гелиос балансировочный станок</t>
+          <t>конус для балансировки колес</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>160</v>
+        <v>16</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -3782,23 +3781,23 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировочные станки (общие)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-sivik</t>
+          <t>/catalog/balansirovochnye-stanki</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>приспособление для балансировки колес</t>
+          <t>пробаланс шиномонтажное оборудование</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>159</v>
+        <v>16</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -3807,7 +3806,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировка в составе шиномонтажного оборудования</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -3819,11 +3818,11 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>балансир для колес</t>
+          <t>сбмп 40 л балансировочный станок</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>158</v>
+        <v>16</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -3844,11 +3843,11 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>балансировочный станок nordberg 4523c</t>
+          <t>балансировочный станок hofmann</t>
         </is>
       </c>
       <c r="B35" t="n">
-        <v>153</v>
+        <v>16</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -3862,18 +3861,18 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-nordberg</t>
+          <t>/catalog/balansirovochnye-stanki</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>балансировочный станок сивик альфа</t>
+          <t>балансировочный станок es 750</t>
         </is>
       </c>
       <c r="B36" t="n">
-        <v>147</v>
+        <v>15</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -3882,23 +3881,23 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировочные станки (общие)</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-sivik</t>
+          <t>/catalog/balansirovochnye-stanki</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>балансировочный станок beissbarth</t>
+          <t>балансировочный станок россвик</t>
         </is>
       </c>
       <c r="B37" t="n">
-        <v>145</v>
+        <v>15</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -3919,11 +3918,11 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>аппарат для балансировки колес</t>
+          <t>ручной балансировочный станок для колес</t>
         </is>
       </c>
       <c r="B38" t="n">
-        <v>138</v>
+        <v>15</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -3944,11 +3943,11 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>лазерный балансировочный станок</t>
+          <t>балансировочный станок с виброконтролем</t>
         </is>
       </c>
       <c r="B39" t="n">
-        <v>133</v>
+        <v>14</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -3969,11 +3968,11 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>сивик стандарт балансировочный станок</t>
+          <t>балансировочный станок sivik galaxy plus</t>
         </is>
       </c>
       <c r="B40" t="n">
-        <v>131</v>
+        <v>13</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -3994,11 +3993,11 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>балансировочный станок ает</t>
+          <t>балансир для колес</t>
         </is>
       </c>
       <c r="B41" t="n">
-        <v>126</v>
+        <v>13</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -4019,11 +4018,11 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>балансировочный станок техносоюз</t>
+          <t>ts 500 балансировочный станок</t>
         </is>
       </c>
       <c r="B42" t="n">
-        <v>125</v>
+        <v>13</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -4032,7 +4031,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировочные станки (общие)</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -4044,11 +4043,11 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>оборудование для балансировки колес</t>
+          <t>балансировочный станок сивик альфа</t>
         </is>
       </c>
       <c r="B43" t="n">
-        <v>125</v>
+        <v>12</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -4057,23 +4056,23 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировочные станки по брендам</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>/catalog/balansirovochnye-stanki/brand-sivik</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>спутник люкс балансировочный станок</t>
+          <t>пб 02м балансировочный станок</t>
         </is>
       </c>
       <c r="B44" t="n">
-        <v>117</v>
+        <v>12</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -4082,7 +4081,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировочные станки (общие)</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -4094,11 +4093,11 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>балансировочный станок сивик мастер</t>
+          <t>балансировочный станок civic</t>
         </is>
       </c>
       <c r="B45" t="n">
-        <v>117</v>
+        <v>12</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
@@ -4107,23 +4106,23 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировочные станки (общие)</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-sivik</t>
+          <t>/catalog/balansirovochnye-stanki</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>балансировочный станок сивик галакси плюс</t>
+          <t>вес балансировочного станка для шиномонтажа</t>
         </is>
       </c>
       <c r="B46" t="n">
-        <v>116</v>
+        <v>11</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
@@ -4132,23 +4131,23 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировка в составе шиномонтажного оборудования</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-sivik</t>
+          <t>/catalog/balansirovochnye-stanki</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>балансировочный станок sicam</t>
+          <t>стенд для балансировки колес купить</t>
         </is>
       </c>
       <c r="B47" t="n">
-        <v>113</v>
+        <v>11</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
@@ -4157,7 +4156,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировочные станки (общие)</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -4169,11 +4168,11 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>балансировочный станок sivik сбмк 60</t>
+          <t>балансировочный станок сторм лс1 01</t>
         </is>
       </c>
       <c r="B48" t="n">
-        <v>110</v>
+        <v>11</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
@@ -4187,27 +4186,27 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-sivik</t>
+          <t>/catalog/balansirovochnye-stanki/brand-storm</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>как настроить балансировочный станок</t>
+          <t>балансировочный станок россвик вт 62</t>
         </is>
       </c>
       <c r="B49" t="n">
-        <v>109</v>
+        <v>11</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Информационный</t>
+          <t>Коммерческий</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировочные станки по брендам</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -4219,11 +4218,11 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>балансировочный станок для шиномонтажа сивик</t>
+          <t>балансировочный станок для грузовых автомобилей</t>
         </is>
       </c>
       <c r="B50" t="n">
-        <v>103</v>
+        <v>11</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
@@ -4232,23 +4231,23 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировочные станки для грузовых</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-sivik</t>
+          <t>/catalog/balansirovochnye-stanki-dlya-gruzovyh-avtomobilej</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>балансировочный станок nordberg 4523</t>
+          <t>es 750 балансировочный станок для легковых авто</t>
         </is>
       </c>
       <c r="B51" t="n">
-        <v>102</v>
+        <v>10</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
@@ -4257,23 +4256,23 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировочные станки для легковых</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-nordberg</t>
+          <t>/catalog/balansirovochnye-stanki-dlya-legkovyh-avtomobilej</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>сбмп 40 л балансировочный станок</t>
+          <t>балансировочный станок alpha luxe сбмп 40 л</t>
         </is>
       </c>
       <c r="B52" t="n">
-        <v>101</v>
+        <v>10</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
@@ -4294,11 +4293,11 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>cb1930b балансировочный станок</t>
+          <t>krw240 балансировочный станок</t>
         </is>
       </c>
       <c r="B53" t="n">
-        <v>100</v>
+        <v>9</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
@@ -4319,11 +4318,11 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>балансировочный станок wiederkraft</t>
+          <t>балансировочный станок galaxy plus</t>
         </is>
       </c>
       <c r="B54" t="n">
-        <v>94</v>
+        <v>9</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
@@ -4344,11 +4343,11 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>балансировочный станок sivik galaxy plus</t>
+          <t>купить балансировочный станок в новосибирске</t>
         </is>
       </c>
       <c r="B55" t="n">
-        <v>93</v>
+        <v>9</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
@@ -4357,23 +4356,23 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировочные станки (общие)</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-sivik</t>
+          <t>/catalog/balansirovochnye-stanki</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>балансировочный станок hofmann geodyna</t>
+          <t>купить балансировочный станок в москве</t>
         </is>
       </c>
       <c r="B56" t="n">
-        <v>92</v>
+        <v>9</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
@@ -4382,7 +4381,7 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировочные станки (общие)</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
@@ -4394,11 +4393,11 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>балансировочный станок es 750</t>
+          <t>балансировочный станок с прижимным роликом</t>
         </is>
       </c>
       <c r="B57" t="n">
-        <v>87</v>
+        <v>9</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
@@ -4419,36 +4418,36 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>станок для балансировки колес купить</t>
+          <t>грузик для калибровки балансировочного станка</t>
         </is>
       </c>
       <c r="B58" t="n">
-        <v>84</v>
+        <v>9</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Коммерческий</t>
+          <t>Информационный</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировочные грузики</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>/catalog/gruziki-balansirovochnye</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>купить балансировочный станок цена</t>
+          <t>балансировочный станок крафт</t>
         </is>
       </c>
       <c r="B59" t="n">
-        <v>83</v>
+        <v>9</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
@@ -4469,11 +4468,11 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>балансировочный станок sivik sputnik</t>
+          <t>балансировочный станок для грузовых колес</t>
         </is>
       </c>
       <c r="B60" t="n">
-        <v>83</v>
+        <v>9</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
@@ -4482,23 +4481,23 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировочные станки для грузовых</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-sivik</t>
+          <t>/catalog/balansirovochnye-stanki-dlya-gruzovyh-avtomobilej</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>балансировочный станок станкоимпорт</t>
+          <t>балансировочный станок для шиномонтажа nordberg</t>
         </is>
       </c>
       <c r="B61" t="n">
-        <v>80</v>
+        <v>9</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
@@ -4512,18 +4511,18 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>/catalog/balansirovochnye-stanki/brand-nordberg</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>грузовой балансировочный станок купить</t>
+          <t>балансировочный станок нордберг 4523n1</t>
         </is>
       </c>
       <c r="B62" t="n">
-        <v>79</v>
+        <v>8</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
@@ -4532,32 +4531,32 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Балансировочные станки для грузовых</t>
+          <t>Балансировочные станки по брендам</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki-dlya-gruzovyh-avtomobilej</t>
+          <t>/catalog/balansirovochnye-stanki/brand-nordberg</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>как выставить балансировочный станок</t>
+          <t>балансировочный станок гелиос</t>
         </is>
       </c>
       <c r="B63" t="n">
-        <v>75</v>
+        <v>8</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Информационный</t>
+          <t>Коммерческий</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировочные станки по брендам</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -4569,11 +4568,11 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>балансировочные грузики для литых дисков</t>
+          <t>балансировочный станок beissbarth</t>
         </is>
       </c>
       <c r="B64" t="n">
-        <v>71</v>
+        <v>8</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
@@ -4582,23 +4581,23 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Балансировочные грузики</t>
+          <t>Балансировочные станки по брендам</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>/catalog/gruziki-balansirovochnye</t>
+          <t>/catalog/balansirovochnye-stanki</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>балансировочный станок для грузовых колес</t>
+          <t>sivik stellar балансировочный станок</t>
         </is>
       </c>
       <c r="B65" t="n">
-        <v>70</v>
+        <v>8</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
@@ -4607,23 +4606,23 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Балансировочные станки для грузовых</t>
+          <t>Балансировочные станки по брендам</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki-dlya-gruzovyh-avtomobilej</t>
+          <t>/catalog/balansirovochnye-stanki/brand-sivik</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>балансировочный станок сикам</t>
+          <t>балансировочный станок хантер с роликом</t>
         </is>
       </c>
       <c r="B66" t="n">
-        <v>67</v>
+        <v>8</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
@@ -4632,27 +4631,27 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировочные станки по брендам</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>/catalog/balansirovochnye-stanki/brand-hunterengineering</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>как установить балансировочный станок</t>
+          <t>балансировочный станок сикам</t>
         </is>
       </c>
       <c r="B67" t="n">
-        <v>67</v>
+        <v>8</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Информационный</t>
+          <t>Коммерческий</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -4669,11 +4668,11 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>балансировочный станок сивик спутник</t>
+          <t>купить балансировочный станок для шиномонтажа сивик</t>
         </is>
       </c>
       <c r="B68" t="n">
-        <v>65</v>
+        <v>7</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
@@ -4694,11 +4693,11 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>балансировочный станок спутник стандарт</t>
+          <t>спутник люкс балансировочный станок</t>
         </is>
       </c>
       <c r="B69" t="n">
-        <v>65</v>
+        <v>7</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
@@ -4719,11 +4718,11 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>балансировочный станок нордберг 4523n1</t>
+          <t>балансировочный станок nordberg 4525</t>
         </is>
       </c>
       <c r="B70" t="n">
-        <v>64</v>
+        <v>7</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
@@ -4744,36 +4743,36 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>балансировочный станок для грузовых автомобилей</t>
+          <t>как настроить балансировочный станок для колес автомобиля</t>
         </is>
       </c>
       <c r="B71" t="n">
-        <v>63</v>
+        <v>7</v>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Коммерческий</t>
+          <t>Информационный</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Балансировочные станки для грузовых</t>
+          <t>Балансировочные станки (общие)</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki-dlya-gruzovyh-avtomobilej</t>
+          <t>/catalog/balansirovochnye-stanki</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>устройство для балансировки колес</t>
+          <t>как пользоваться балансировочным станком для колес</t>
         </is>
       </c>
       <c r="B72" t="n">
-        <v>62</v>
+        <v>7</v>
       </c>
       <c r="C72" t="inlineStr">
         <is>
@@ -4794,11 +4793,11 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>балансировочный станок нордберг 4523с</t>
+          <t>балансировочный станок станкоимпорт st 200a</t>
         </is>
       </c>
       <c r="B73" t="n">
-        <v>61</v>
+        <v>7</v>
       </c>
       <c r="C73" t="inlineStr">
         <is>
@@ -4812,18 +4811,18 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-nordberg</t>
+          <t>/catalog/balansirovochnye-stanki</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>балансировочный станок rossvik vt 61</t>
+          <t>автоматический балансировочный станок для шиномонтажа</t>
         </is>
       </c>
       <c r="B74" t="n">
-        <v>60</v>
+        <v>6</v>
       </c>
       <c r="C74" t="inlineStr">
         <is>
@@ -4832,7 +4831,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Автоматические балансировочные станки</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -4844,11 +4843,11 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>прибор для балансировки колес</t>
+          <t>адаптер для балансировки колес</t>
         </is>
       </c>
       <c r="B75" t="n">
-        <v>59</v>
+        <v>6</v>
       </c>
       <c r="C75" t="inlineStr">
         <is>
@@ -4869,20 +4868,20 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>оборудование для шиномонтаж и балансировка</t>
+          <t>как настроить балансировочный станок</t>
         </is>
       </c>
       <c r="B76" t="n">
-        <v>57</v>
+        <v>6</v>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Коммерческий</t>
+          <t>Информационный</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Балансировка в составе шиномонтажного оборудования</t>
+          <t>Балансировочные станки (общие)</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -4894,11 +4893,11 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>балансировочный станок trommelberg cb1930b</t>
+          <t>лазерный балансировочный станок</t>
         </is>
       </c>
       <c r="B77" t="n">
-        <v>57</v>
+        <v>6</v>
       </c>
       <c r="C77" t="inlineStr">
         <is>
@@ -4907,7 +4906,7 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировочные станки (общие)</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
@@ -4919,11 +4918,11 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>балансировочный станок galaxy сбмп 60 3d</t>
+          <t>станок для балансировки колес легковых автомобилей</t>
         </is>
       </c>
       <c r="B78" t="n">
-        <v>56</v>
+        <v>6</v>
       </c>
       <c r="C78" t="inlineStr">
         <is>
@@ -4932,23 +4931,23 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировочные станки для легковых</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>/catalog/balansirovochnye-stanki-dlya-legkovyh-avtomobilej</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>китайский балансировочный станок</t>
+          <t>балансировочный станок техносоюз</t>
         </is>
       </c>
       <c r="B79" t="n">
-        <v>55</v>
+        <v>6</v>
       </c>
       <c r="C79" t="inlineStr">
         <is>
@@ -4957,7 +4956,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировочные станки по брендам</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -4969,11 +4968,11 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>стенд балансировочный грузовой</t>
+          <t>балансировочный станок sivik сбмк 60</t>
         </is>
       </c>
       <c r="B80" t="n">
-        <v>53</v>
+        <v>6</v>
       </c>
       <c r="C80" t="inlineStr">
         <is>
@@ -4982,32 +4981,32 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Балансировочные станки для грузовых</t>
+          <t>Балансировочные станки по брендам</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki-dlya-gruzovyh-avtomobilej</t>
+          <t>/catalog/balansirovochnye-stanki/brand-sivik</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>как правильно установить балансировочный станок</t>
+          <t>аппарат для шиномонтажа и балансировки цена</t>
         </is>
       </c>
       <c r="B81" t="n">
-        <v>51</v>
+        <v>6</v>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Информационный</t>
+          <t>Коммерческий</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировка в составе шиномонтажного оборудования</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -5019,11 +5018,11 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>балансировочный станок для шиномонтажа цена</t>
+          <t>сторм балансировочный станок официальный сайт</t>
         </is>
       </c>
       <c r="B82" t="n">
-        <v>50</v>
+        <v>6</v>
       </c>
       <c r="C82" t="inlineStr">
         <is>
@@ -5032,23 +5031,23 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Балансировка в составе шиномонтажного оборудования</t>
+          <t>Балансировочные станки по брендам</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>/catalog/balansirovochnye-stanki/brand-storm</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>станок для динамической балансировки</t>
+          <t>балансировочный станок nordberg 4523</t>
         </is>
       </c>
       <c r="B83" t="n">
-        <v>48</v>
+        <v>5</v>
       </c>
       <c r="C83" t="inlineStr">
         <is>
@@ -5057,23 +5056,23 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировочные станки по брендам</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>/catalog/balansirovochnye-stanki/brand-nordberg</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>фланцевый адаптер для балансировки колес</t>
+          <t>балансировочный станок для шиномонтажа грузовых автомобилей</t>
         </is>
       </c>
       <c r="B84" t="n">
-        <v>45</v>
+        <v>5</v>
       </c>
       <c r="C84" t="inlineStr">
         <is>
@@ -5082,23 +5081,23 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировочные станки для грузовых</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>/catalog/balansirovochnye-stanki-dlya-gruzovyh-avtomobilej</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>купить балансировочный станок для шиномонтажа сивик</t>
+          <t>балансировочный станок автоматический</t>
         </is>
       </c>
       <c r="B85" t="n">
-        <v>45</v>
+        <v>5</v>
       </c>
       <c r="C85" t="inlineStr">
         <is>
@@ -5107,23 +5106,23 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Автоматические балансировочные станки</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-sivik</t>
+          <t>/catalog/balansirovochnye-stanki</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>балансировочный станок sputnik сбмк 60</t>
+          <t>балансировочный бисер для колес</t>
         </is>
       </c>
       <c r="B86" t="n">
-        <v>44</v>
+        <v>5</v>
       </c>
       <c r="C86" t="inlineStr">
         <is>
@@ -5144,11 +5143,11 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>горизонтальный балансировочный станок</t>
+          <t>балансировщик колес цена</t>
         </is>
       </c>
       <c r="B87" t="n">
-        <v>44</v>
+        <v>5</v>
       </c>
       <c r="C87" t="inlineStr">
         <is>
@@ -5169,11 +5168,11 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>сивик старт балансировочный станок купить</t>
+          <t>балансировка колес стоимость аппарата</t>
         </is>
       </c>
       <c r="B88" t="n">
-        <v>44</v>
+        <v>5</v>
       </c>
       <c r="C88" t="inlineStr">
         <is>
@@ -5182,23 +5181,23 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировочные станки (общие)</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-sivik</t>
+          <t>/catalog/balansirovochnye-stanki</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>challenger 3 балансировочный станок</t>
+          <t>грузовой балансировочный станок сивик</t>
         </is>
       </c>
       <c r="B89" t="n">
-        <v>43</v>
+        <v>5</v>
       </c>
       <c r="C89" t="inlineStr">
         <is>
@@ -5207,23 +5206,23 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировочные станки для грузовых</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>/catalog/balansirovochnye-stanki-dlya-gruzovyh-avtomobilej</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>балансировочный станок kraftwell krw242</t>
+          <t>станок для динамической балансировки</t>
         </is>
       </c>
       <c r="B90" t="n">
-        <v>43</v>
+        <v>5</v>
       </c>
       <c r="C90" t="inlineStr">
         <is>
@@ -5232,7 +5231,7 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировочные станки (общие)</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
@@ -5244,11 +5243,11 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>балансировочный станок сивик сбмп 60 3d</t>
+          <t>оборудование для балансировки колес легковых автомобилей</t>
         </is>
       </c>
       <c r="B91" t="n">
-        <v>41</v>
+        <v>4</v>
       </c>
       <c r="C91" t="inlineStr">
         <is>
@@ -5257,23 +5256,23 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировочные станки для легковых</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-sivik</t>
+          <t>/catalog/balansirovochnye-stanki-dlya-legkovyh-avtomobilej</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>станок для балансировки колес легковых автомобилей</t>
+          <t>балансировочный станок ает</t>
         </is>
       </c>
       <c r="B92" t="n">
-        <v>40</v>
+        <v>4</v>
       </c>
       <c r="C92" t="inlineStr">
         <is>
@@ -5282,23 +5281,23 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Балансировочные станки для легковых</t>
+          <t>Балансировочные станки (общие)</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki-dlya-legkovyh-avtomobilej</t>
+          <t>/catalog/balansirovochnye-stanki</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>балансировочный станок сторм лс1 01</t>
+          <t>самоклеющиеся балансировочные грузики</t>
         </is>
       </c>
       <c r="B93" t="n">
-        <v>39</v>
+        <v>4</v>
       </c>
       <c r="C93" t="inlineStr">
         <is>
@@ -5307,23 +5306,23 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировочные грузики</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-storm</t>
+          <t>/catalog/gruziki-balansirovochnye</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>sivik stellar балансировочный станок</t>
+          <t>балансировочный станок nordberg 4524c</t>
         </is>
       </c>
       <c r="B94" t="n">
-        <v>38</v>
+        <v>4</v>
       </c>
       <c r="C94" t="inlineStr">
         <is>
@@ -5337,18 +5336,18 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-sivik</t>
+          <t>/catalog/balansirovochnye-stanki/brand-nordberg</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>балансировочный станок с виброконтролем</t>
+          <t>волчок для балансировки колес</t>
         </is>
       </c>
       <c r="B95" t="n">
-        <v>38</v>
+        <v>4</v>
       </c>
       <c r="C95" t="inlineStr">
         <is>
@@ -5369,11 +5368,11 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>балансировочный станок для грузового шиномонтажа</t>
+          <t>стоимость оборудования для шиномонтажа и балансировки цена</t>
         </is>
       </c>
       <c r="B96" t="n">
-        <v>38</v>
+        <v>4</v>
       </c>
       <c r="C96" t="inlineStr">
         <is>
@@ -5382,23 +5381,23 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Балансировочные станки для грузовых</t>
+          <t>Балансировка в составе шиномонтажного оборудования</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki-dlya-gruzovyh-avtomobilej</t>
+          <t>/catalog/balansirovochnye-stanki</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>балансировочный станок нордберг 4524с</t>
+          <t>балансировочный станок с виброконтролем купить</t>
         </is>
       </c>
       <c r="B97" t="n">
-        <v>37</v>
+        <v>4</v>
       </c>
       <c r="C97" t="inlineStr">
         <is>
@@ -5407,23 +5406,23 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировочные станки (общие)</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-nordberg</t>
+          <t>/catalog/balansirovochnye-stanki</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>балансировочный станок nordberg 4524c</t>
+          <t>станок балансировочный легковой</t>
         </is>
       </c>
       <c r="B98" t="n">
-        <v>37</v>
+        <v>3</v>
       </c>
       <c r="C98" t="inlineStr">
         <is>
@@ -5432,23 +5431,23 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировочные станки для легковых</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-nordberg</t>
+          <t>/catalog/balansirovochnye-stanki-dlya-legkovyh-avtomobilej</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>балансировочный станок nordberg 4525</t>
+          <t>балансировочный станок шторм</t>
         </is>
       </c>
       <c r="B99" t="n">
-        <v>37</v>
+        <v>3</v>
       </c>
       <c r="C99" t="inlineStr">
         <is>
@@ -5457,23 +5456,23 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировочные станки (общие)</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-nordberg</t>
+          <t>/catalog/balansirovochnye-stanki</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>балансировочный стенд hofmann geodyna</t>
+          <t>стенд для динамической балансировки</t>
         </is>
       </c>
       <c r="B100" t="n">
-        <v>36</v>
+        <v>3</v>
       </c>
       <c r="C100" t="inlineStr">
         <is>
@@ -5482,7 +5481,7 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировочные станки (общие)</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
@@ -5494,11 +5493,11 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>балансировочный станок для шиномонтажа nordberg</t>
+          <t>грузовой балансировочный станок купить</t>
         </is>
       </c>
       <c r="B101" t="n">
-        <v>36</v>
+        <v>3</v>
       </c>
       <c r="C101" t="inlineStr">
         <is>
@@ -5507,12 +5506,12 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировочные станки для грузовых</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-nordberg</t>
+          <t>/catalog/balansirovochnye-stanki-dlya-gruzovyh-avtomobilej</t>
         </is>
       </c>
     </row>
@@ -5520,70 +5519,4 @@
   <autoFilter ref="A1:E101"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="150" customWidth="1" min="1" max="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Сайт: t-ind.ru. Направления: шиномонтажное оборудование; балансировочные станки (по 100 запросов).</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Источник: выгрузки органической выдачи по региону Москва и по региону GRU (2 CSV), 36 761 строка, 31 490 уникальных запросов.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Частотность — «Базовая частотность» (WS) из выгрузки, максимум по двум регионам. Запросы с нулевой базовой или точной частотностью исключены.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Дубли по порядку слов/транслиту (sivik = сивик) схлопнуты, оставлен вариант с большей частотностью.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Исключены: услуги шиномонтажа (рядом, цены, круглосуточно), вакансии, б/у, «своими руками», инструкции, размеры шин, одиночные слова-прилагательные без предмета.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Интент определён по маркерам: купить/цена/заказ → коммерческий; как/что такое/выбрать → информационный; товарный запрос без маркеров → коммерческий.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Целевая страница — ближайший по смыслу существующий раздел каталога (проверен по URL в выгрузке); для брендов — страница бренда.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Semantic core: replace clusters and target pages with new clustering
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016UEhV6w824sjkUhMCvDZb2
</commit_message>
<xml_diff>
--- a/semantic_core_t-ind.ru.xlsx
+++ b/semantic_core_t-ind.ru.xlsx
@@ -480,12 +480,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование (общие)</t>
+          <t>Шиномонтаж: оборудование (общие)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnoe-oborudovanie</t>
         </is>
       </c>
     </row>
@@ -505,12 +505,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки</t>
+          <t>Шиномонтаж: станки (общие)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki</t>
         </is>
       </c>
     </row>
@@ -530,12 +530,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование (общие)</t>
+          <t>Шиномонтаж: оборудование (общие)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnoe-oborudovanie</t>
         </is>
       </c>
     </row>
@@ -555,12 +555,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Ручные шиномонтажные станки</t>
+          <t>Шиномонтаж: ручные станки</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej</t>
+          <t>(создать) /catalog/shinomontazhnye-stanki/vid-ruchnoj</t>
         </is>
       </c>
     </row>
@@ -580,12 +580,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки</t>
+          <t>Шиномонтаж: станки (общие)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki</t>
         </is>
       </c>
     </row>
@@ -605,12 +605,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование по брендам</t>
+          <t>Шиномонтаж: бренд Sivik</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie/brand-sivik</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnoe-oborudovanie/brand-sivik</t>
         </is>
       </c>
     </row>
@@ -630,12 +630,12 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование по брендам</t>
+          <t>Шиномонтаж: бренд Sivik</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie/brand-sivik</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnoe-oborudovanie/brand-sivik</t>
         </is>
       </c>
     </row>
@@ -655,12 +655,12 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Комплекты и инструмент для шиномонтажа</t>
+          <t>Шиномонтаж: комплекты оборудования</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>/catalog/komplekty-shinomontazhnogo-oborudovaniya</t>
+          <t>https://t-ind.ru/catalog/komplekty-shinomontazhnogo-oborudovaniya</t>
         </is>
       </c>
     </row>
@@ -680,12 +680,12 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Ручные шиномонтажные станки</t>
+          <t>Шиномонтаж: ручные станки</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej</t>
+          <t>(создать) /catalog/shinomontazhnye-stanki/vid-ruchnoj</t>
         </is>
       </c>
     </row>
@@ -705,12 +705,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Комплекты и инструмент для шиномонтажа</t>
+          <t>Шиномонтаж: комплекты оборудования</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>/catalog/komplekty-shinomontazhnogo-oborudovaniya</t>
+          <t>https://t-ind.ru/catalog/komplekty-shinomontazhnogo-oborudovaniya</t>
         </is>
       </c>
     </row>
@@ -730,12 +730,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование по брендам</t>
+          <t>Шиномонтаж: бренд Sivik</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie/brand-sivik</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnoe-oborudovanie/brand-sivik</t>
         </is>
       </c>
     </row>
@@ -755,12 +755,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки для грузовых</t>
+          <t>Шиномонтаж: станки для грузовых</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki-dlya-gruzovyh-avtomobilej</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki-dlya-gruzovyh-avtomobilej</t>
         </is>
       </c>
     </row>
@@ -780,12 +780,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки для легковых</t>
+          <t>Шиномонтаж: станки для легковых</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej</t>
         </is>
       </c>
     </row>
@@ -805,12 +805,12 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки для грузовых</t>
+          <t>Шиномонтаж: станки для грузовых</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki-dlya-gruzovyh-avtomobilej</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki-dlya-gruzovyh-avtomobilej</t>
         </is>
       </c>
     </row>
@@ -830,12 +830,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование по брендам</t>
+          <t>Шиномонтаж: прочие бренды (Rossvik, Феникс, Сибек, WDK, Пробаланс)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnoe-oborudovanie</t>
         </is>
       </c>
     </row>
@@ -855,12 +855,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки для легковых</t>
+          <t>Шиномонтаж: станки для легковых</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej</t>
         </is>
       </c>
     </row>
@@ -880,12 +880,12 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование по брендам</t>
+          <t>Шиномонтаж: бренд Nordberg</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie/brand-nordberg</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki/brand-nordberg</t>
         </is>
       </c>
     </row>
@@ -905,12 +905,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Ручные шиномонтажные станки</t>
+          <t>Шиномонтаж: ручные станки</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej</t>
+          <t>(создать) /catalog/shinomontazhnye-stanki/vid-ruchnoj</t>
         </is>
       </c>
     </row>
@@ -930,12 +930,12 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование по брендам</t>
+          <t>Шиномонтаж: бренд Hunter</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie/brand-hunterengineering</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnoe-oborudovanie/brand-hunterengineering</t>
         </is>
       </c>
     </row>
@@ -955,12 +955,12 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки для легковых</t>
+          <t>Шиномонтаж: станки для легковых</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej</t>
         </is>
       </c>
     </row>
@@ -980,12 +980,12 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Ручные шиномонтажные станки</t>
+          <t>Шиномонтаж: ручные станки</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej</t>
+          <t>(создать) /catalog/shinomontazhnye-stanki/vid-ruchnoj</t>
         </is>
       </c>
     </row>
@@ -1005,12 +1005,12 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование (общие)</t>
+          <t>Шиномонтаж: аксессуар «третья рука»</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>https://t-ind.ru/catalog/tretya-ruka-dlya-shinomontazhnyh-stankov</t>
         </is>
       </c>
     </row>
@@ -1030,12 +1030,12 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование (общие)</t>
+          <t>Шиномонтаж: региональные запросы</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnoe-oborudovanie</t>
         </is>
       </c>
     </row>
@@ -1055,12 +1055,12 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки</t>
+          <t>Шиномонтаж: станки (общие)</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki</t>
         </is>
       </c>
     </row>
@@ -1080,12 +1080,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Комплекты и инструмент для шиномонтажа</t>
+          <t>Шиномонтаж: комплекты оборудования</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>/catalog/komplekty-shinomontazhnogo-oborudovaniya</t>
+          <t>https://t-ind.ru/catalog/komplekty-shinomontazhnogo-oborudovaniya</t>
         </is>
       </c>
     </row>
@@ -1105,12 +1105,12 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Автоматические шиномонтажные станки</t>
+          <t>Шиномонтаж: автоматические станки</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki/vid-avtomaticheskij</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki/vid-avtomaticheskij</t>
         </is>
       </c>
     </row>
@@ -1130,12 +1130,12 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки для легковых</t>
+          <t>Шиномонтаж: станки для легковых</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej</t>
         </is>
       </c>
     </row>
@@ -1155,12 +1155,12 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки для грузовых</t>
+          <t>Шиномонтаж: станки для грузовых</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki-dlya-gruzovyh-avtomobilej</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki-dlya-gruzovyh-avtomobilej</t>
         </is>
       </c>
     </row>
@@ -1180,12 +1180,12 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование по брендам</t>
+          <t>Шиномонтаж: бренд Hofmann</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki/brand-hofmann</t>
         </is>
       </c>
     </row>
@@ -1205,12 +1205,12 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование (общие)</t>
+          <t>Шиномонтаж: региональные запросы</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnoe-oborudovanie</t>
         </is>
       </c>
     </row>
@@ -1230,12 +1230,12 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование (общие)</t>
+          <t>Шиномонтаж: оборудование (общие)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnoe-oborudovanie</t>
         </is>
       </c>
     </row>
@@ -1255,12 +1255,12 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование по брендам</t>
+          <t>Шиномонтаж: бренд Nordberg</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie/brand-nordberg</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki/brand-nordberg</t>
         </is>
       </c>
     </row>
@@ -1280,12 +1280,12 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Комплекты и инструмент для шиномонтажа</t>
+          <t>Шиномонтаж: комплекты оборудования</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>/catalog/komplekty-shinomontazhnogo-oborudovaniya</t>
+          <t>https://t-ind.ru/catalog/komplekty-shinomontazhnogo-oborudovaniya</t>
         </is>
       </c>
     </row>
@@ -1305,12 +1305,12 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Комплекты и инструмент для шиномонтажа</t>
+          <t>Шиномонтаж: комплекты оборудования</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>/catalog/komplekty-shinomontazhnogo-oborudovaniya</t>
+          <t>https://t-ind.ru/catalog/komplekty-shinomontazhnogo-oborudovaniya</t>
         </is>
       </c>
     </row>
@@ -1330,12 +1330,12 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование (общие)</t>
+          <t>Шиномонтаж: станки 220 В</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki/setv-220</t>
         </is>
       </c>
     </row>
@@ -1355,12 +1355,12 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование (общие)</t>
+          <t>Шиномонтаж: оборудование (общие)</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnoe-oborudovanie</t>
         </is>
       </c>
     </row>
@@ -1380,12 +1380,12 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки для грузовых</t>
+          <t>Шиномонтаж: станки для грузовых</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki-dlya-gruzovyh-avtomobilej</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki-dlya-gruzovyh-avtomobilej</t>
         </is>
       </c>
     </row>
@@ -1405,12 +1405,12 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки для легковых</t>
+          <t>Шиномонтаж: станки для легковых</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej</t>
         </is>
       </c>
     </row>
@@ -1430,12 +1430,12 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование (общие)</t>
+          <t>Шиномонтаж: оборудование (общие)</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnoe-oborudovanie</t>
         </is>
       </c>
     </row>
@@ -1455,12 +1455,12 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки для грузовых</t>
+          <t>Шиномонтаж: станки для грузовых</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki-dlya-gruzovyh-avtomobilej</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki-dlya-gruzovyh-avtomobilej</t>
         </is>
       </c>
     </row>
@@ -1480,12 +1480,12 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование (общие)</t>
+          <t>Шиномонтаж: аксессуар «третья рука»</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>https://t-ind.ru/catalog/tretya-ruka-dlya-shinomontazhnyh-stankov</t>
         </is>
       </c>
     </row>
@@ -1505,12 +1505,12 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки для грузовых</t>
+          <t>Шиномонтаж: станки для грузовых</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki-dlya-gruzovyh-avtomobilej</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki-dlya-gruzovyh-avtomobilej</t>
         </is>
       </c>
     </row>
@@ -1530,12 +1530,12 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки</t>
+          <t>Шиномонтаж: станки (синонимы «разбортовочный/бортировочный»)</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki</t>
         </is>
       </c>
     </row>
@@ -1555,12 +1555,12 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование по брендам</t>
+          <t>Шиномонтаж: Nordberg 4638</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie/brand-nordberg</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki/brand-nordberg</t>
         </is>
       </c>
     </row>
@@ -1580,12 +1580,12 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки для легковых</t>
+          <t>Шиномонтаж: станки для легковых</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej</t>
         </is>
       </c>
     </row>
@@ -1605,12 +1605,12 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование (общие)</t>
+          <t>Шиномонтаж: прочие бренды (Rossvik, Феникс, Сибек, WDK, Пробаланс)</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnoe-oborudovanie</t>
         </is>
       </c>
     </row>
@@ -1630,12 +1630,12 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование по брендам</t>
+          <t>Шиномонтаж: бренд Kraftwell</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki/brand-kraftwell</t>
         </is>
       </c>
     </row>
@@ -1655,12 +1655,12 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование (общие)</t>
+          <t>Шиномонтаж: оборудование (общие)</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnoe-oborudovanie</t>
         </is>
       </c>
     </row>
@@ -1680,12 +1680,12 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование (общие)</t>
+          <t>Шиномонтаж: оборудование (общие)</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnoe-oborudovanie</t>
         </is>
       </c>
     </row>
@@ -1705,12 +1705,12 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Комплекты и инструмент для шиномонтажа</t>
+          <t>Шиномонтаж: комплекты оборудования</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>/catalog/komplekty-shinomontazhnogo-oborudovaniya</t>
+          <t>https://t-ind.ru/catalog/komplekty-shinomontazhnogo-oborudovaniya</t>
         </is>
       </c>
     </row>
@@ -1730,12 +1730,12 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки для легковых</t>
+          <t>Шиномонтаж: станки 220 В</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki/setv-220</t>
         </is>
       </c>
     </row>
@@ -1755,12 +1755,12 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование по брендам</t>
+          <t>Шиномонтаж: модели Sivik (КС 302/402/508)</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie/brand-sivik</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej/brand-sivik</t>
         </is>
       </c>
     </row>
@@ -1780,12 +1780,12 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки для легковых</t>
+          <t>Шиномонтаж: станки для легковых</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej</t>
         </is>
       </c>
     </row>
@@ -1805,12 +1805,12 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование по брендам</t>
+          <t>Шиномонтаж: Nordberg 4638</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie/brand-nordberg</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki/brand-nordberg</t>
         </is>
       </c>
     </row>
@@ -1830,12 +1830,12 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки</t>
+          <t>Шиномонтаж: бренд EQFS</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej/brand-eqfs</t>
         </is>
       </c>
     </row>
@@ -1855,12 +1855,12 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование (общие)</t>
+          <t>Шиномонтаж: региональные запросы</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnoe-oborudovanie</t>
         </is>
       </c>
     </row>
@@ -1880,12 +1880,12 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование по брендам</t>
+          <t>Шиномонтаж: модели Sivik (КС 302/402/508)</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie/brand-sivik</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej/brand-sivik</t>
         </is>
       </c>
     </row>
@@ -1905,12 +1905,12 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки</t>
+          <t>Шиномонтаж: станки (общие)</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki</t>
         </is>
       </c>
     </row>
@@ -1930,12 +1930,12 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки</t>
+          <t>Шиномонтаж: станки с третьей рукой</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki/tretyaruka-da</t>
         </is>
       </c>
     </row>
@@ -1955,12 +1955,12 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Автоматические шиномонтажные станки</t>
+          <t>Шиномонтаж: модели Sivik (КС 302/402/508)</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki/vid-avtomaticheskij</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej/brand-sivik</t>
         </is>
       </c>
     </row>
@@ -1980,12 +1980,12 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование по брендам</t>
+          <t>Шиномонтаж: бренд Kraftwell</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki/brand-kraftwell</t>
         </is>
       </c>
     </row>
@@ -2005,12 +2005,12 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование по брендам</t>
+          <t>Шиномонтаж: бренд Hunter</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie/brand-hunterengineering</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnoe-oborudovanie/brand-hunterengineering</t>
         </is>
       </c>
     </row>
@@ -2030,12 +2030,12 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование (общие)</t>
+          <t>Шиномонтаж: станки (общие)</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki</t>
         </is>
       </c>
     </row>
@@ -2055,12 +2055,12 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки</t>
+          <t>Шиномонтаж: станки с третьей рукой</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki/tretyaruka-da</t>
         </is>
       </c>
     </row>
@@ -2080,12 +2080,12 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Комплекты и инструмент для шиномонтажа</t>
+          <t>Шиномонтаж: комплекты оборудования</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>/catalog/komplekty-shinomontazhnogo-oborudovaniya</t>
+          <t>https://t-ind.ru/catalog/komplekty-shinomontazhnogo-oborudovaniya</t>
         </is>
       </c>
     </row>
@@ -2105,12 +2105,12 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки</t>
+          <t>Шиномонтаж: станки (общие)</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki</t>
         </is>
       </c>
     </row>
@@ -2130,12 +2130,12 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки</t>
+          <t>Шиномонтаж: прочие модели (Hofmann Monty, M&amp;B, ГШС)</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnoe-oborudovanie</t>
         </is>
       </c>
     </row>
@@ -2155,12 +2155,12 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки для грузовых</t>
+          <t>Шиномонтаж: станки для грузовых</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki-dlya-gruzovyh-avtomobilej</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki-dlya-gruzovyh-avtomobilej</t>
         </is>
       </c>
     </row>
@@ -2180,12 +2180,12 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование по брендам</t>
+          <t>Шиномонтаж: бренд Sivik</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie/brand-sivik</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnoe-oborudovanie/brand-sivik</t>
         </is>
       </c>
     </row>
@@ -2205,12 +2205,12 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование по брендам</t>
+          <t>Шиномонтаж: бренд Hofmann</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki/brand-hofmann</t>
         </is>
       </c>
     </row>
@@ -2230,12 +2230,12 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование по брендам</t>
+          <t>Шиномонтаж: бренд Hunter</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie/brand-hunterengineering</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnoe-oborudovanie/brand-hunterengineering</t>
         </is>
       </c>
     </row>
@@ -2255,12 +2255,12 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки для легковых</t>
+          <t>Шиномонтаж: ручные станки</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej</t>
+          <t>(создать) /catalog/shinomontazhnye-stanki/vid-ruchnoj</t>
         </is>
       </c>
     </row>
@@ -2280,12 +2280,12 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование по брендам</t>
+          <t>Шиномонтаж: бренд Hofmann</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki/brand-hofmann</t>
         </is>
       </c>
     </row>
@@ -2305,12 +2305,12 @@
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки</t>
+          <t>Шиномонтаж: станки 220 В</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki/setv-220</t>
         </is>
       </c>
     </row>
@@ -2330,12 +2330,12 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование (общие)</t>
+          <t>Шиномонтаж: информационные (устройство станка, список оборудования)</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>(создать) /stati/ustrojstvo-shinomontazhnogo-stanka</t>
         </is>
       </c>
     </row>
@@ -2355,12 +2355,12 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Комплекты и инструмент для шиномонтажа</t>
+          <t>Шиномонтаж: комплекты оборудования</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>/catalog/komplekty-shinomontazhnogo-oborudovaniya</t>
+          <t>https://t-ind.ru/catalog/komplekty-shinomontazhnogo-oborudovaniya</t>
         </is>
       </c>
     </row>
@@ -2380,12 +2380,12 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование по брендам</t>
+          <t>Шиномонтаж: бренд Sicam</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki/brand-sicam</t>
         </is>
       </c>
     </row>
@@ -2405,12 +2405,12 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование по брендам</t>
+          <t>Шиномонтаж: бренд Hofmann</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki/brand-hofmann</t>
         </is>
       </c>
     </row>
@@ -2430,12 +2430,12 @@
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Автоматические шиномонтажные станки</t>
+          <t>Шиномонтаж: модели Sivik (КС 302/402/508)</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki/vid-avtomaticheskij</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej/brand-sivik</t>
         </is>
       </c>
     </row>
@@ -2455,12 +2455,12 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование (общие)</t>
+          <t>Шиномонтаж: оборудование (общие)</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnoe-oborudovanie</t>
         </is>
       </c>
     </row>
@@ -2480,12 +2480,12 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование (общие)</t>
+          <t>Шиномонтаж: информационные (устройство станка, список оборудования)</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>(создать) /stati/ustrojstvo-shinomontazhnogo-stanka</t>
         </is>
       </c>
     </row>
@@ -2505,12 +2505,12 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование (общие)</t>
+          <t>Шиномонтаж: прочие бренды (Rossvik, Феникс, Сибек, WDK, Пробаланс)</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnoe-oborudovanie</t>
         </is>
       </c>
     </row>
@@ -2530,12 +2530,12 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование по брендам</t>
+          <t>Шиномонтаж: аксессуар «третья рука»</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie/brand-sivik</t>
+          <t>https://t-ind.ru/catalog/tretya-ruka-dlya-shinomontazhnyh-stankov</t>
         </is>
       </c>
     </row>
@@ -2555,12 +2555,12 @@
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование (общие)</t>
+          <t>Шиномонтаж: бренд Техновектор</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnoe-oborudovanie/brand-tehnovektor</t>
         </is>
       </c>
     </row>
@@ -2580,12 +2580,12 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование (общие)</t>
+          <t>Шиномонтаж: запчасти для станков</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>https://t-ind.ru/catalog/rashodnye-materialy-dlya-shinomontazhnogo-oborudovaniya</t>
         </is>
       </c>
     </row>
@@ -2605,12 +2605,12 @@
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование по брендам</t>
+          <t>Шиномонтаж: бренд Beissbarth</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki/brand-beissbarth</t>
         </is>
       </c>
     </row>
@@ -2630,12 +2630,12 @@
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки</t>
+          <t>Шиномонтаж: региональные запросы</t>
         </is>
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnoe-oborudovanie</t>
         </is>
       </c>
     </row>
@@ -2655,12 +2655,12 @@
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование (общие)</t>
+          <t>Шиномонтаж: региональные запросы</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnoe-oborudovanie</t>
         </is>
       </c>
     </row>
@@ -2680,12 +2680,12 @@
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование (общие)</t>
+          <t>Шиномонтаж: оборудование (общие)</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnoe-oborudovanie</t>
         </is>
       </c>
     </row>
@@ -2705,12 +2705,12 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование по брендам</t>
+          <t>Шиномонтаж: бренд Storm</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie/brand-storm</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnoe-oborudovanie/brand-storm</t>
         </is>
       </c>
     </row>
@@ -2730,12 +2730,12 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки</t>
+          <t>Шиномонтаж: прочие бренды (Rossvik, Феникс, Сибек, WDK, Пробаланс)</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnoe-oborudovanie</t>
         </is>
       </c>
     </row>
@@ -2755,12 +2755,12 @@
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование (общие)</t>
+          <t>Шиномонтаж: запчасти для станков</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>https://t-ind.ru/catalog/rashodnye-materialy-dlya-shinomontazhnogo-oborudovaniya</t>
         </is>
       </c>
     </row>
@@ -2780,12 +2780,12 @@
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки</t>
+          <t>Шиномонтаж: станки (синонимы «разбортовочный/бортировочный»)</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki</t>
         </is>
       </c>
     </row>
@@ -2805,12 +2805,12 @@
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Комплекты и инструмент для шиномонтажа</t>
+          <t>Шиномонтаж: комплекты оборудования</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>/catalog/komplekty-shinomontazhnogo-oborudovaniya</t>
+          <t>https://t-ind.ru/catalog/komplekty-shinomontazhnogo-oborudovaniya</t>
         </is>
       </c>
     </row>
@@ -2830,12 +2830,12 @@
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование (общие)</t>
+          <t>Шиномонтаж: запчасти для станков</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>https://t-ind.ru/catalog/rashodnye-materialy-dlya-shinomontazhnogo-oborudovaniya</t>
         </is>
       </c>
     </row>
@@ -2855,12 +2855,12 @@
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование (общие)</t>
+          <t>Шиномонтаж: ручной инструмент</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>https://t-ind.ru/catalog/ruchnoj-instrument-dlya-shinomontazha</t>
         </is>
       </c>
     </row>
@@ -2880,12 +2880,12 @@
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Комплекты и инструмент для шиномонтажа</t>
+          <t>Шиномонтаж: комплекты оборудования</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>/catalog/komplekty-shinomontazhnogo-oborudovaniya</t>
+          <t>https://t-ind.ru/catalog/komplekty-shinomontazhnogo-oborudovaniya</t>
         </is>
       </c>
     </row>
@@ -2905,12 +2905,12 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Шиномонтажное оборудование по брендам</t>
+          <t>Шиномонтаж: прочие модели (Hofmann Monty, M&amp;B, ГШС)</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnoe-oborudovanie</t>
         </is>
       </c>
     </row>
@@ -2930,12 +2930,12 @@
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки</t>
+          <t>Шиномонтаж: прочие модели (Hofmann Monty, M&amp;B, ГШС)</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnoe-oborudovanie</t>
         </is>
       </c>
     </row>
@@ -2955,12 +2955,12 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Шиномонтажные станки</t>
+          <t>Шиномонтаж: модели Sivik (КС 302/402/508)</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>/catalog/shinomontazhnye-stanki</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej/brand-sivik</t>
         </is>
       </c>
     </row>
@@ -2980,12 +2980,12 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировка: станки (общие)</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki</t>
         </is>
       </c>
     </row>
@@ -3005,12 +3005,12 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>Балансировка в составе шиномонтажного оборудования</t>
+          <t>Балансировка: станки (общие)</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki</t>
         </is>
       </c>
     </row>
@@ -3030,12 +3030,12 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Балансировка в составе шиномонтажного оборудования</t>
+          <t>Балансировка: станки (общие)</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki</t>
         </is>
       </c>
     </row>
@@ -3055,12 +3055,12 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировка: бренд Sivik</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-sivik</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-sivik</t>
         </is>
       </c>
     </row>
@@ -3080,12 +3080,12 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Балансировочные станки для грузовых</t>
+          <t>Балансировка: для грузовых</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki-dlya-gruzovyh-avtomobilej</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki-dlya-gruzovyh-avtomobilej</t>
         </is>
       </c>
     </row>
@@ -3105,12 +3105,12 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировка: станки (общие)</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki</t>
         </is>
       </c>
     </row>
@@ -3130,12 +3130,12 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировка: станки (общие)</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki</t>
         </is>
       </c>
     </row>
@@ -3155,12 +3155,12 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировка: бренд Nordberg</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-nordberg</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-nordberg</t>
         </is>
       </c>
     </row>
@@ -3180,12 +3180,12 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировка: станки (общие)</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki</t>
         </is>
       </c>
     </row>
@@ -3205,12 +3205,12 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировка: бренд Hunter</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-hunterengineering</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-hunterengineering</t>
         </is>
       </c>
     </row>
@@ -3230,12 +3230,12 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировка: бренд Sivik</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-sivik</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-sivik</t>
         </is>
       </c>
     </row>
@@ -3255,12 +3255,12 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировка: станки (общие)</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki</t>
         </is>
       </c>
     </row>
@@ -3280,12 +3280,12 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировка: станки с нагрузочным/прижимным роликом</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>(создать) /catalog/balansirovochnye-stanki/s-rolikom</t>
         </is>
       </c>
     </row>
@@ -3305,12 +3305,12 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировка: бренд Sivik</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-sivik</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-sivik</t>
         </is>
       </c>
     </row>
@@ -3330,12 +3330,12 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировка: Sivik Galaxy Plus</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-sivik</t>
+          <t>(создать) /catalog/balansirovochnye-stanki/sivik-galaxy-plus</t>
         </is>
       </c>
     </row>
@@ -3355,12 +3355,12 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировка: прочие серии Sivik (Start, Stellar, СБМК 60, Спутник)</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-sivik</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-sivik</t>
         </is>
       </c>
     </row>
@@ -3380,12 +3380,12 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировка: станки (общие)</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki</t>
         </is>
       </c>
     </row>
@@ -3405,12 +3405,12 @@
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировка: бренд Storm</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-storm</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-storm</t>
         </is>
       </c>
     </row>
@@ -3430,12 +3430,12 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировка: Sivik Gelios</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-sivik</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-sivik</t>
         </is>
       </c>
     </row>
@@ -3455,12 +3455,12 @@
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировка: модели Nordberg 4523/4524/4525</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-nordberg</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-nordberg</t>
         </is>
       </c>
     </row>
@@ -3480,12 +3480,12 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Балансировка в составе шиномонтажного оборудования</t>
+          <t>Балансировка: станки (общие)</t>
         </is>
       </c>
       <c r="E122" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki</t>
         </is>
       </c>
     </row>
@@ -3505,12 +3505,12 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировка: модели EQFS ES 750 / Kraftwell KRW</t>
         </is>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-kraftwell</t>
         </is>
       </c>
     </row>
@@ -3530,12 +3530,12 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировка: станки (общие)</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki</t>
         </is>
       </c>
     </row>
@@ -3555,12 +3555,12 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировка: бренд Sicam</t>
         </is>
       </c>
       <c r="E125" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-sicam</t>
         </is>
       </c>
     </row>
@@ -3580,12 +3580,12 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Балансировочные станки для легковых</t>
+          <t>Балансировка: станки (общие)</t>
         </is>
       </c>
       <c r="E126" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki-dlya-legkovyh-avtomobilej</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki</t>
         </is>
       </c>
     </row>
@@ -3605,12 +3605,12 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировка: бренд Trommelberg</t>
         </is>
       </c>
       <c r="E127" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-trommelberg</t>
         </is>
       </c>
     </row>
@@ -3630,12 +3630,12 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировка: Sivik Galaxy Plus</t>
         </is>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-sivik</t>
+          <t>(создать) /catalog/balansirovochnye-stanki/sivik-galaxy-plus</t>
         </is>
       </c>
     </row>
@@ -3655,12 +3655,12 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Балансировка в составе шиномонтажного оборудования</t>
+          <t>Шиномонтаж: прочие бренды (Rossvik, Феникс, Сибек, WDK, Пробаланс)</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnoe-oborudovanie</t>
         </is>
       </c>
     </row>
@@ -3680,12 +3680,12 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировка: Sivik Alpha Luxe (СБМП 40 Л)</t>
         </is>
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-sivik</t>
         </is>
       </c>
     </row>
@@ -3705,12 +3705,12 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировка: бренды Beissbarth / Hofmann</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-beissbarth</t>
         </is>
       </c>
     </row>
@@ -3730,12 +3730,12 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировка: модели EQFS ES 750 / Kraftwell KRW</t>
         </is>
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-kraftwell</t>
         </is>
       </c>
     </row>
@@ -3755,12 +3755,12 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировка: бренд Rossvik</t>
         </is>
       </c>
       <c r="E133" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-rossvik</t>
         </is>
       </c>
     </row>
@@ -3780,12 +3780,12 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировка: ручные станки</t>
         </is>
       </c>
       <c r="E134" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/vid-ruchnojvvod</t>
         </is>
       </c>
     </row>
@@ -3805,12 +3805,12 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировка: станки с виброконтролем</t>
         </is>
       </c>
       <c r="E135" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>(создать) /catalog/balansirovochnye-stanki/s-vibrokontrolem</t>
         </is>
       </c>
     </row>
@@ -3830,12 +3830,12 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировка: Sivik Galaxy Plus</t>
         </is>
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-sivik</t>
+          <t>(создать) /catalog/balansirovochnye-stanki/sivik-galaxy-plus</t>
         </is>
       </c>
     </row>
@@ -3855,12 +3855,12 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировка: станки (общие)</t>
         </is>
       </c>
       <c r="E137" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki</t>
         </is>
       </c>
     </row>
@@ -3880,12 +3880,12 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировка: прочие бренды и модели</t>
         </is>
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/brands</t>
         </is>
       </c>
     </row>
@@ -3905,12 +3905,12 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировка: Sivik Alpha Luxe (СБМП 40 Л)</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-sivik</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-sivik</t>
         </is>
       </c>
     </row>
@@ -3930,12 +3930,12 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировка: прочие бренды и модели</t>
         </is>
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/brands</t>
         </is>
       </c>
     </row>
@@ -3955,12 +3955,12 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировка: бренд Sivik</t>
         </is>
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-sivik</t>
         </is>
       </c>
     </row>
@@ -3980,12 +3980,12 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировка: станки (общие)</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki</t>
         </is>
       </c>
     </row>
@@ -4005,12 +4005,12 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировка: бренд Storm</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-storm</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-storm</t>
         </is>
       </c>
     </row>
@@ -4030,12 +4030,12 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировка: бренд Rossvik</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-rossvik</t>
         </is>
       </c>
     </row>
@@ -4055,12 +4055,12 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>Балансировочные станки для грузовых</t>
+          <t>Балансировка: для грузовых</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki-dlya-gruzovyh-avtomobilej</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki-dlya-gruzovyh-avtomobilej</t>
         </is>
       </c>
     </row>
@@ -4080,12 +4080,12 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>Балансировочные станки для легковых</t>
+          <t>Балансировка: модели EQFS ES 750 / Kraftwell KRW</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki-dlya-legkovyh-avtomobilej</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-kraftwell</t>
         </is>
       </c>
     </row>
@@ -4105,12 +4105,12 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировка: Sivik Alpha Luxe (СБМП 40 Л)</t>
         </is>
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-sivik</t>
         </is>
       </c>
     </row>
@@ -4130,12 +4130,12 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировка: модели EQFS ES 750 / Kraftwell KRW</t>
         </is>
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-kraftwell</t>
         </is>
       </c>
     </row>
@@ -4155,12 +4155,12 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировка: Sivik Galaxy Plus</t>
         </is>
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>(создать) /catalog/balansirovochnye-stanki/sivik-galaxy-plus</t>
         </is>
       </c>
     </row>
@@ -4180,12 +4180,12 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировка: региональные запросы</t>
         </is>
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki</t>
         </is>
       </c>
     </row>
@@ -4205,12 +4205,12 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировка: региональные запросы</t>
         </is>
       </c>
       <c r="E151" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki</t>
         </is>
       </c>
     </row>
@@ -4230,12 +4230,12 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировка: станки с нагрузочным/прижимным роликом</t>
         </is>
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>(создать) /catalog/balansirovochnye-stanki/s-rolikom</t>
         </is>
       </c>
     </row>
@@ -4255,12 +4255,12 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировка: прочие бренды и модели</t>
         </is>
       </c>
       <c r="E153" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/brands</t>
         </is>
       </c>
     </row>
@@ -4280,12 +4280,12 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>Балансировочные станки для грузовых</t>
+          <t>Балансировка: для грузовых</t>
         </is>
       </c>
       <c r="E154" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki-dlya-gruzovyh-avtomobilej</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki-dlya-gruzovyh-avtomobilej</t>
         </is>
       </c>
     </row>
@@ -4305,12 +4305,12 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировка: бренд Nordberg</t>
         </is>
       </c>
       <c r="E155" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-nordberg</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-nordberg</t>
         </is>
       </c>
     </row>
@@ -4330,12 +4330,12 @@
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировка: модели Nordberg 4523/4524/4525</t>
         </is>
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-nordberg</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-nordberg</t>
         </is>
       </c>
     </row>
@@ -4355,12 +4355,12 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировка: Sivik Gelios</t>
         </is>
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-sivik</t>
         </is>
       </c>
     </row>
@@ -4380,12 +4380,12 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировка: бренды Beissbarth / Hofmann</t>
         </is>
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-beissbarth</t>
         </is>
       </c>
     </row>
@@ -4405,12 +4405,12 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировка: прочие серии Sivik (Start, Stellar, СБМК 60, Спутник)</t>
         </is>
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-sivik</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-sivik</t>
         </is>
       </c>
     </row>
@@ -4430,12 +4430,12 @@
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировка: станки с нагрузочным/прижимным роликом</t>
         </is>
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-hunterengineering</t>
+          <t>(создать) /catalog/balansirovochnye-stanki/s-rolikom</t>
         </is>
       </c>
     </row>
@@ -4455,12 +4455,12 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировка: бренд Sicam</t>
         </is>
       </c>
       <c r="E161" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-sicam</t>
         </is>
       </c>
     </row>
@@ -4480,12 +4480,12 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировка: бренд Sivik</t>
         </is>
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-sivik</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-sivik</t>
         </is>
       </c>
     </row>
@@ -4505,12 +4505,12 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировка: прочие серии Sivik (Start, Stellar, СБМК 60, Спутник)</t>
         </is>
       </c>
       <c r="E163" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-sivik</t>
         </is>
       </c>
     </row>
@@ -4530,12 +4530,12 @@
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировка: модели Nordberg 4523/4524/4525</t>
         </is>
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-nordberg</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-nordberg</t>
         </is>
       </c>
     </row>
@@ -4555,12 +4555,12 @@
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировка: инструкции (настройка, эксплуатация, установка)</t>
         </is>
       </c>
       <c r="E165" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>(создать) /stati/kak-nastroit-balansirovochnyj-stanok</t>
         </is>
       </c>
     </row>
@@ -4580,12 +4580,12 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировка: инструкции (настройка, эксплуатация, установка)</t>
         </is>
       </c>
       <c r="E166" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>(создать) /stati/kak-nastroit-balansirovochnyj-stanok</t>
         </is>
       </c>
     </row>
@@ -4605,12 +4605,12 @@
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировка: прочие бренды и модели</t>
         </is>
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/brands</t>
         </is>
       </c>
     </row>
@@ -4630,12 +4630,12 @@
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>Автоматические балансировочные станки</t>
+          <t>Балансировка: станки (общие)</t>
         </is>
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki</t>
         </is>
       </c>
     </row>
@@ -4655,12 +4655,12 @@
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировка: инструкции (настройка, эксплуатация, установка)</t>
         </is>
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>(создать) /stati/kak-nastroit-balansirovochnyj-stanok</t>
         </is>
       </c>
     </row>
@@ -4680,12 +4680,12 @@
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировка: общий каталог</t>
         </is>
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki</t>
         </is>
       </c>
     </row>
@@ -4705,12 +4705,12 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>Балансировочные станки для легковых</t>
+          <t>Балансировка: станки (общие)</t>
         </is>
       </c>
       <c r="E171" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki-dlya-legkovyh-avtomobilej</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki</t>
         </is>
       </c>
     </row>
@@ -4730,12 +4730,12 @@
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировка: прочие бренды и модели</t>
         </is>
       </c>
       <c r="E172" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/brands</t>
         </is>
       </c>
     </row>
@@ -4755,12 +4755,12 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировка: прочие серии Sivik (Start, Stellar, СБМК 60, Спутник)</t>
         </is>
       </c>
       <c r="E173" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-sivik</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-sivik</t>
         </is>
       </c>
     </row>
@@ -4780,12 +4780,12 @@
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>Балансировка в составе шиномонтажного оборудования</t>
+          <t>Шиномонтаж: оборудование (общие)</t>
         </is>
       </c>
       <c r="E174" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnoe-oborudovanie</t>
         </is>
       </c>
     </row>
@@ -4805,12 +4805,12 @@
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировка: бренд Storm</t>
         </is>
       </c>
       <c r="E175" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-storm</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-storm</t>
         </is>
       </c>
     </row>
@@ -4830,12 +4830,12 @@
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировка: модели Nordberg 4523/4524/4525</t>
         </is>
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-nordberg</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-nordberg</t>
         </is>
       </c>
     </row>
@@ -4855,12 +4855,12 @@
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>Балансировочные станки для грузовых</t>
+          <t>Балансировка: для грузовых</t>
         </is>
       </c>
       <c r="E177" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki-dlya-gruzovyh-avtomobilej</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki-dlya-gruzovyh-avtomobilej</t>
         </is>
       </c>
     </row>
@@ -4880,12 +4880,12 @@
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>Автоматические балансировочные станки</t>
+          <t>Балансировка: станки (общие)</t>
         </is>
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki</t>
         </is>
       </c>
     </row>
@@ -4905,12 +4905,12 @@
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировка: станки (общие)</t>
         </is>
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki</t>
         </is>
       </c>
     </row>
@@ -4930,12 +4930,12 @@
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировка: станки (общие)</t>
         </is>
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki</t>
         </is>
       </c>
     </row>
@@ -4955,12 +4955,12 @@
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>Балансировочные станки для грузовых</t>
+          <t>Балансировка: для грузовых</t>
         </is>
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki-dlya-gruzovyh-avtomobilej</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki-dlya-gruzovyh-avtomobilej</t>
         </is>
       </c>
     </row>
@@ -4980,12 +4980,12 @@
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировка: динамическая балансировка (стенд/станок)</t>
         </is>
       </c>
       <c r="E182" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki</t>
         </is>
       </c>
     </row>
@@ -5005,12 +5005,12 @@
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>Балансировочные станки для легковых</t>
+          <t>Балансировка: станки (общие)</t>
         </is>
       </c>
       <c r="E183" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki-dlya-legkovyh-avtomobilej</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki</t>
         </is>
       </c>
     </row>
@@ -5030,12 +5030,12 @@
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировка: станки (общие)</t>
         </is>
       </c>
       <c r="E184" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki</t>
         </is>
       </c>
     </row>
@@ -5055,12 +5055,12 @@
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировка: модели Nordberg 4523/4524/4525</t>
         </is>
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-nordberg</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-nordberg</t>
         </is>
       </c>
     </row>
@@ -5080,12 +5080,12 @@
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>Балансировка в составе шиномонтажного оборудования</t>
+          <t>Шиномонтаж: оборудование (общие)</t>
         </is>
       </c>
       <c r="E186" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnoe-oborudovanie</t>
         </is>
       </c>
     </row>
@@ -5105,12 +5105,12 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировка: станки с виброконтролем</t>
         </is>
       </c>
       <c r="E187" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>(создать) /catalog/balansirovochnye-stanki/s-vibrokontrolem</t>
         </is>
       </c>
     </row>
@@ -5130,12 +5130,12 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>Балансировочные станки для легковых</t>
+          <t>Балансировка: станки (общие)</t>
         </is>
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki-dlya-legkovyh-avtomobilej</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki</t>
         </is>
       </c>
     </row>
@@ -5155,12 +5155,12 @@
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировка: бренд Storm</t>
         </is>
       </c>
       <c r="E189" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-storm</t>
         </is>
       </c>
     </row>
@@ -5180,12 +5180,12 @@
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировка: динамическая балансировка (стенд/станок)</t>
         </is>
       </c>
       <c r="E190" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki</t>
         </is>
       </c>
     </row>
@@ -5205,12 +5205,12 @@
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>Балансировочные станки для грузовых</t>
+          <t>Балансировка: для грузовых</t>
         </is>
       </c>
       <c r="E191" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki-dlya-gruzovyh-avtomobilej</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki-dlya-gruzovyh-avtomobilej</t>
         </is>
       </c>
     </row>
@@ -5230,12 +5230,12 @@
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировка: прочие бренды и модели</t>
         </is>
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/brands</t>
         </is>
       </c>
     </row>
@@ -5255,12 +5255,12 @@
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировка: станки (общие)</t>
         </is>
       </c>
       <c r="E193" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki</t>
         </is>
       </c>
     </row>
@@ -5280,12 +5280,12 @@
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>Балансировка в составе шиномонтажного оборудования</t>
+          <t>Балансировка: инструкции (настройка, эксплуатация, установка)</t>
         </is>
       </c>
       <c r="E194" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>(создать) /stati/kak-nastroit-balansirovochnyj-stanok</t>
         </is>
       </c>
     </row>
@@ -5305,12 +5305,12 @@
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>Балансировочные станки для легковых</t>
+          <t>Балансировка: станки (общие)</t>
         </is>
       </c>
       <c r="E195" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki-dlya-legkovyh-avtomobilej</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki</t>
         </is>
       </c>
     </row>
@@ -5330,12 +5330,12 @@
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировка: станки (общие)</t>
         </is>
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki</t>
         </is>
       </c>
     </row>
@@ -5355,12 +5355,12 @@
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>Балансировочные станки (общие)</t>
+          <t>Балансировка: станки (общие)</t>
         </is>
       </c>
       <c r="E197" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki</t>
         </is>
       </c>
     </row>
@@ -5380,12 +5380,12 @@
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>Балансировка в составе шиномонтажного оборудования</t>
+          <t>Шиномонтаж: оборудование (общие)</t>
         </is>
       </c>
       <c r="E198" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnoe-oborudovanie</t>
         </is>
       </c>
     </row>
@@ -5405,12 +5405,12 @@
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>Балансировка в составе шиномонтажного оборудования</t>
+          <t>Шиномонтаж: прочие бренды (Rossvik, Феникс, Сибек, WDK, Пробаланс)</t>
         </is>
       </c>
       <c r="E199" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki</t>
+          <t>https://t-ind.ru/catalog/shinomontazhnoe-oborudovanie</t>
         </is>
       </c>
     </row>
@@ -5430,12 +5430,12 @@
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>Балансировочные станки по брендам</t>
+          <t>Балансировка: бренд Hunter</t>
         </is>
       </c>
       <c r="E200" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki/brand-hunterengineering</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-hunterengineering</t>
         </is>
       </c>
     </row>
@@ -5455,12 +5455,12 @@
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>Балансировочные станки для грузовых</t>
+          <t>Балансировка: для грузовых</t>
         </is>
       </c>
       <c r="E201" t="inlineStr">
         <is>
-          <t>/catalog/balansirovochnye-stanki-dlya-gruzovyh-avtomobilej</t>
+          <t>https://t-ind.ru/catalog/balansirovochnye-stanki-dlya-gruzovyh-avtomobilej</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Clustering: add target URLs and page types, product cards for model queries
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016UEhV6w824sjkUhMCvDZb2
</commit_message>
<xml_diff>
--- a/semantic_core_t-ind.ru.xlsx
+++ b/semantic_core_t-ind.ru.xlsx
@@ -1560,7 +1560,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki/brand-nordberg</t>
+          <t>https://t-ind.ru/products/shinomontazhnyj-stanok-poluavtomat-nordberg-4638e_220v</t>
         </is>
       </c>
     </row>
@@ -1760,7 +1760,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej/brand-sivik</t>
+          <t>https://t-ind.ru/products/shinomontazhnyj-stanok-sivik-ks-302a-legkovoj-poluavtomaticheskij-220-v</t>
         </is>
       </c>
     </row>
@@ -1810,7 +1810,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki/brand-nordberg</t>
+          <t>https://t-ind.ru/products/shinomontazhnyj-stanok-poluavtomat-nordberg-4638e_220v</t>
         </is>
       </c>
     </row>
@@ -1885,7 +1885,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej/brand-sivik</t>
+          <t>https://t-ind.ru/products/shinomontazhnyj-stanok-sivik-ks-402a-pro-legkovoj-avtomaticheskij-220-v</t>
         </is>
       </c>
     </row>
@@ -1960,7 +1960,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej/brand-sivik</t>
+          <t>https://t-ind.ru/products/shinomontazhnyj-stanok-legkovoj-sivik-ks-508a-pro-superavtomat-invertornyj-220v-s-tretej-rukoj</t>
         </is>
       </c>
     </row>
@@ -2435,7 +2435,7 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej/brand-sivik</t>
+          <t>https://t-ind.ru/products/shinomontazhnyj-stanok-sivik-ks-402a-pro-legkovoj-avtomaticheskij-380-v</t>
         </is>
       </c>
     </row>
@@ -2910,7 +2910,7 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>https://t-ind.ru/catalog/shinomontazhnoe-oborudovanie</t>
+          <t>https://t-ind.ru/products/shinomontazhnyj-stanok-legkovoj-hofmann-monty-3300-20-smart-gp-plus-avtomaticheskij-s-tretej-rukoj-380v</t>
         </is>
       </c>
     </row>
@@ -2960,7 +2960,7 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>https://t-ind.ru/catalog/shinomontazhnye-stanki-dlya-legkovyh-avtomobilej/brand-sivik</t>
+          <t>https://t-ind.ru/products/shinomontazhnyj-stanok-sivik-ks-302a-legkovoj-poluavtomaticheskij-220-v</t>
         </is>
       </c>
     </row>
@@ -3335,7 +3335,7 @@
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>(создать) /catalog/balansirovochnye-stanki/sivik-galaxy-plus</t>
+          <t>https://t-ind.ru/products/balansirovochnyj-stanok-sivik-galaxy-plus-sbmp-603d-l-seryj-legkovoj-avtomaticheskij-220v</t>
         </is>
       </c>
     </row>
@@ -3435,7 +3435,7 @@
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-sivik</t>
+          <t>https://t-ind.ru/products/balansirovochnyj-stanok-sivik-gelios-sbmp-603d-plus-uztlu-legkovoj-avtomaticheskij-220-v</t>
         </is>
       </c>
     </row>
@@ -3460,7 +3460,7 @@
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-nordberg</t>
+          <t>https://t-ind.ru/products/balansirovochnyj-stanok-dlya-gruzovyhlegkovyh-avtomobilej-nordberg-4523c-poluavtomat</t>
         </is>
       </c>
     </row>
@@ -3510,7 +3510,7 @@
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-kraftwell</t>
+          <t>https://t-ind.ru/products/balansirovochnyj-stanok-dlya-gruzovyhlegkovyh-avtomobilej-kraftwell-krw242-avtomaticheskij</t>
         </is>
       </c>
     </row>
@@ -3635,7 +3635,7 @@
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>(создать) /catalog/balansirovochnye-stanki/sivik-galaxy-plus</t>
+          <t>https://t-ind.ru/products/balansirovochnyj-stanok-sivik-galaxy-plus-sbmp-603d-l-seryj-legkovoj-avtomaticheskij-220v</t>
         </is>
       </c>
     </row>
@@ -3685,7 +3685,7 @@
       </c>
       <c r="E130" t="inlineStr">
         <is>
-          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-sivik</t>
+          <t>https://t-ind.ru/products/balansirovochnyj-stanok-sivik-alpha-luxe-sbmp-40-l-sinij-legkovoj-poluavtomaticheskij-220v</t>
         </is>
       </c>
     </row>
@@ -3735,7 +3735,7 @@
       </c>
       <c r="E132" t="inlineStr">
         <is>
-          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-kraftwell</t>
+          <t>https://t-ind.ru/products/balansirovochnyj-stanok-eqfs-es-750-legkovoj-dlya-motokoles-avtomat-220v</t>
         </is>
       </c>
     </row>
@@ -3835,7 +3835,7 @@
       </c>
       <c r="E136" t="inlineStr">
         <is>
-          <t>(создать) /catalog/balansirovochnye-stanki/sivik-galaxy-plus</t>
+          <t>https://t-ind.ru/products/balansirovochnyj-stanok-sivik-galaxy-plus-sbmp-603d-l-seryj-legkovoj-avtomaticheskij-220v</t>
         </is>
       </c>
     </row>
@@ -3885,7 +3885,7 @@
       </c>
       <c r="E138" t="inlineStr">
         <is>
-          <t>https://t-ind.ru/brands</t>
+          <t>https://t-ind.ru/products/balansirovochnyj-stanok-tehnosoyuz-ts-500-legkovoj-poluavtomaticheskij-220v</t>
         </is>
       </c>
     </row>
@@ -3910,7 +3910,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-sivik</t>
+          <t>https://t-ind.ru/products/balansirovochnyj-stanok-sivik-alpha-luxe-sbmp-40-l-sinij-legkovoj-poluavtomaticheskij-220v</t>
         </is>
       </c>
     </row>
@@ -4035,7 +4035,7 @@
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-rossvik</t>
+          <t>https://t-ind.ru/products/balansirovochnyj-stanok-rossvik-vt-62-new-legkovoj-dlya-motokoles-poluavtomaticheskij-220v</t>
         </is>
       </c>
     </row>
@@ -4085,7 +4085,7 @@
       </c>
       <c r="E146" t="inlineStr">
         <is>
-          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-kraftwell</t>
+          <t>https://t-ind.ru/products/balansirovochnyj-stanok-eqfs-es-750-legkovoj-dlya-motokoles-avtomat-220v</t>
         </is>
       </c>
     </row>
@@ -4110,7 +4110,7 @@
       </c>
       <c r="E147" t="inlineStr">
         <is>
-          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-sivik</t>
+          <t>https://t-ind.ru/products/balansirovochnyj-stanok-sivik-alpha-luxe-sbmp-40-l-sinij-legkovoj-poluavtomaticheskij-220v</t>
         </is>
       </c>
     </row>
@@ -4135,7 +4135,7 @@
       </c>
       <c r="E148" t="inlineStr">
         <is>
-          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-kraftwell</t>
+          <t>https://t-ind.ru/products/balansirovochnyj-stanok-dlya-gruzovyhlegkovyh-avtomobilej-kraftwell-krw240-ruchnoj-vvod</t>
         </is>
       </c>
     </row>
@@ -4160,7 +4160,7 @@
       </c>
       <c r="E149" t="inlineStr">
         <is>
-          <t>(создать) /catalog/balansirovochnye-stanki/sivik-galaxy-plus</t>
+          <t>https://t-ind.ru/products/balansirovochnyj-stanok-sivik-galaxy-plus-sbmp-603d-l-seryj-legkovoj-avtomaticheskij-220v</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="E156" t="inlineStr">
         <is>
-          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-nordberg</t>
+          <t>https://t-ind.ru/products/balansirovochnyj-stanok-nordberg-4523n1-poluavtomaticheskij-220-v</t>
         </is>
       </c>
     </row>
@@ -4360,7 +4360,7 @@
       </c>
       <c r="E157" t="inlineStr">
         <is>
-          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-sivik</t>
+          <t>https://t-ind.ru/products/balansirovochnyj-stanok-sivik-gelios-sbmp-603d-plus-uztlu-legkovoj-avtomaticheskij-220-v</t>
         </is>
       </c>
     </row>
@@ -4410,7 +4410,7 @@
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-sivik</t>
+          <t>https://t-ind.ru/products/balansirovochnyj-stanok-sivik-stellar-sbmp-603d-pro-uztlu-legkovoj-avtomaticheskij-220v</t>
         </is>
       </c>
     </row>
@@ -4535,7 +4535,7 @@
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-nordberg</t>
+          <t>https://t-ind.ru/products/balansirovochnyj-stanok-dlya-gruzovyhlegkovyh-avtomobilej-nordberg-4525-poluavtomat</t>
         </is>
       </c>
     </row>
@@ -4610,7 +4610,7 @@
       </c>
       <c r="E167" t="inlineStr">
         <is>
-          <t>https://t-ind.ru/brands</t>
+          <t>https://t-ind.ru/products/balansirovochnyj-stanok-stankoimport-st-200a-legkovoj-poluavtomaticheskij-220-v</t>
         </is>
       </c>
     </row>
@@ -4835,7 +4835,7 @@
       </c>
       <c r="E176" t="inlineStr">
         <is>
-          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-nordberg</t>
+          <t>https://t-ind.ru/products/balansirovochnyj-stanok-nordberg-4523-legkovoj-poluavtomaticheskij-220v</t>
         </is>
       </c>
     </row>
@@ -5060,7 +5060,7 @@
       </c>
       <c r="E185" t="inlineStr">
         <is>
-          <t>https://t-ind.ru/catalog/balansirovochnye-stanki/brand-nordberg</t>
+          <t>https://t-ind.ru/products/balansirovochnyj-stanok-dlya-gruzovyhlegkovyh-avtomobilej-nordberg-4524c-poluavtomat</t>
         </is>
       </c>
     </row>
@@ -5235,7 +5235,7 @@
       </c>
       <c r="E192" t="inlineStr">
         <is>
-          <t>https://t-ind.ru/brands</t>
+          <t>https://t-ind.ru/products/balansirovochnyj-stanok-stankoimport-b200a-legkovoj-dlya-motokoles-ruchnoj-220v</t>
         </is>
       </c>
     </row>

</xml_diff>